<commit_message>
Refine public analyst surface
</commit_message>
<xml_diff>
--- a/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
+++ b/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
@@ -3956,7 +3956,7 @@
       <c r="I5"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Keep the CFR band linked to this audit row at 26/33/40 (central 33). Re-sync the website snapshot's methodology_constants so the live InferredTrajectory band reflects 26/40. Avoid reintroducing the 24/30/40 set or the unsupported 30-50 percent range.</t>
+          <t>Keep the CFR band linked to this audit row at 26/33/40 (central 33). Keep generated snapshot constants, README text, NUMBERS_AUDIT.md, the brief, and the public dataset aligned. Avoid reintroducing the 24/30/40 set or the unsupported 30-50 percent range.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -27657,7 +27657,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Keep the CFR band linked to this audit row at 26/33/40 (central 33). Re-sync the website snapshot's methodology_constants so the live InferredTrajectory band reflects 26/40. Avoid reintroducing the 24/30/40 set or the unsupported 30-50 percent range.</t>
+          <t>Keep the CFR band linked to this audit row at 26/33/40 (central 33). Keep generated snapshot constants, README text, NUMBERS_AUDIT.md, the brief, and the public dataset aligned. Avoid reintroducing the 24/30/40 set or the unsupported 30-50 percent range.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -28196,7 +28196,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>The public BDBV spatial map displays named public geographies, health-zone centroids, corridor endpoints, modeled corridors, and calibration corridors with explicit object role separation; it does not display household-level case GPS coordinates.</t>
+          <t>The public BDBV spatial evidence data separates named public geographies, health-zone centroids, corridor endpoints, modeled corridors, and calibration corridors with explicit object role separation; it does not include household-level case GPS coordinates.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -28211,7 +28211,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>apps/site/app/bdbv-2026/_data/zones.json; WHO Disease Outbreak News item 2026-DON602, 15 May 2026.; apps/site/app/bdbv-2026/_data/snapshots/*.json</t>
+          <t>data/zones.json; WHO Disease Outbreak News item 2026-DON602, 15 May 2026.; data/live-bdbv-2026-output.json</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -28221,7 +28221,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Keep the map inspector focused on role, model use, and public claim audit IDs. If case-level or health-area line-list coordinates become available, add a new spatial object class and public claim audit before displaying them.</t>
+          <t>Keep spatial consumers focused on role, model use, and public claim audit IDs. If case-level or health-area line-list coordinates become available, add a new spatial object class and public claim audit before displaying or exporting them.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">

</xml_diff>

<commit_message>
Clean public reader surface
Focus the public LOVS repository on analyst-facing methods, data, evidence chains, reproducibility gates, and release artifacts. Remove downstream publishing bridge code and harden the public release gate.
</commit_message>
<xml_diff>
--- a/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
+++ b/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
@@ -3956,7 +3956,7 @@
       <c r="I5"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Keep the CFR band linked to this audit row at 26/33/40 (central 33). Re-sync the website snapshot's methodology_constants so the live InferredTrajectory band reflects 26/40. Avoid reintroducing the 24/30/40 set or the unsupported 30-50 percent range.</t>
+          <t>Keep the CFR band linked to this audit row at 26/33/40 (central 33). Keep generated snapshot constants, README text, NUMBERS_AUDIT.md, the brief, and the public dataset aligned. Avoid reintroducing the 24/30/40 set or the unsupported 30-50 percent range.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -27657,7 +27657,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Keep the CFR band linked to this audit row at 26/33/40 (central 33). Re-sync the website snapshot's methodology_constants so the live InferredTrajectory band reflects 26/40. Avoid reintroducing the 24/30/40 set or the unsupported 30-50 percent range.</t>
+          <t>Keep the CFR band linked to this audit row at 26/33/40 (central 33). Keep generated snapshot constants, README text, NUMBERS_AUDIT.md, the brief, and the public dataset aligned. Avoid reintroducing the 24/30/40 set or the unsupported 30-50 percent range.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -28196,7 +28196,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>The public BDBV spatial map displays named public geographies, health-zone centroids, corridor endpoints, modeled corridors, and calibration corridors with explicit object role separation; it does not display household-level case GPS coordinates.</t>
+          <t>The public BDBV spatial evidence data separates named public geographies, health-zone centroids, corridor endpoints, modeled corridors, and calibration corridors with explicit object role separation; it does not include household-level case GPS coordinates.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -28211,7 +28211,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>apps/site/app/bdbv-2026/_data/zones.json; WHO Disease Outbreak News item 2026-DON602, 15 May 2026.; apps/site/app/bdbv-2026/_data/snapshots/*.json</t>
+          <t>data/zones.json; WHO Disease Outbreak News item 2026-DON602, 15 May 2026.; data/live-bdbv-2026-output.json</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -28221,7 +28221,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Keep the map inspector focused on role, model use, and public claim audit IDs. If case-level or health-area line-list coordinates become available, add a new spatial object class and public claim audit before displaying them.</t>
+          <t>Keep spatial consumers focused on role, model use, and public claim audit IDs. If case-level or health-area line-list coordinates become available, add a new spatial object class and public claim audit before displaying or exporting them.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">

</xml_diff>

<commit_message>
Prepare May 22 source-review publication surface
</commit_message>
<xml_diff>
--- a/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
+++ b/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
@@ -2661,7 +2661,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>watch_tier_b_minus</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>claimed_confirmed_fatal_case</t>
+          <t>claimed confirmed fatal case</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2726,17 +2726,17 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>unconfirmed_by_public_health_authority</t>
+          <t>not confirmed by public-health authority</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R25"/>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Promote only if DRC MoH/INRB, WHO, Africa CDC, or CDC publishes South Kivu/Bukavu in confirmed case counts, map, line list, or sitrep with sample date/origin, lab method, health zone, travel history, death status, and epidemiologic link status. An armed-group claim, however widely reported, does not meet this bar on its own.</t>
+          <t>Promote only if DRC MoH/INRB, WHO, Africa CDC, or CDC publishes South Kivu/Bukavu in confirmed case counts, map, line list, or sitrep with sample date/origin, lab method, health zone, travel history, death status, and epidemiologic link status. An armed-group claim, however widely reported, does not meet this bar on its own. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2829,17 +2829,17 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R26"/>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Promote only as policy/travel-monitoring context. Do not promote into case counts, affected-zone geography, or corridor calibration unless CDC publishes count/geography data in the same source.</t>
+          <t>Promote only as policy/travel-monitoring context. Do not promote into case counts, affected-zone geography, or corridor calibration unless CDC publishes count/geography data in the same source. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -2867,7 +2867,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>regional_cross_check_counts_context_only</t>
+          <t>regional cross check counts context only</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2932,17 +2932,17 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R27"/>
@@ -2958,7 +2958,7 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Use ECDC May 21 count values only as cross-check staged observations unless ECDC publishes a primary line-list or explicit correction that supersedes CDC/WHO figures.</t>
+          <t>Use ECDC May 21 count values only as cross-check staged observations unless ECDC publishes a primary line-list or explicit correction that supersedes CDC/WHO figures. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -3035,17 +3035,17 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R28"/>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Promote to staged counts/geography only if the alert contains explicit outbreak figures and a reviewer extracts them with denominator semantics.</t>
+          <t>Promote to staged counts/geography only if the alert contains explicit outbreak figures and a reviewer extracts them with denominator semantics. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -3138,17 +3138,17 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R29"/>
@@ -3164,7 +3164,7 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Keep as readiness context unless WHO AFRO publishes count/geography tables in this source.</t>
+          <t>Keep as readiness context unless WHO AFRO publishes count/geography tables in this source. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3176,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>context_tier_a_minus</t>
+          <t>context tier a minus</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -3241,17 +3241,17 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R30"/>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Keep as response/traveler-monitoring context; do not use as outbreak count input.</t>
+          <t>Keep as response/traveler-monitoring context; do not use as outbreak count input. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>context_tier_b_plus</t>
+          <t>context tier b plus</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3344,17 +3344,17 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>published_context_signal_hash_recorded_bytes</t>
+          <t>published context signal hash recorded bytes</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R31"/>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>risk_and_response_context</t>
+          <t>risk and response context</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3447,17 +3447,17 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>official_who_statement</t>
+          <t>official who statement</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R32"/>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Use for risk-context copy and Uganda transmission-status context; do not promote to zone-attributed count input.</t>
+          <t>Use for risk-context copy and Uganda transmission-status context; do not promote to zone-attributed count input. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -3550,17 +3550,17 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R33"/>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Keep as context-only unless CDC publishes explicit count/geography data in this source and a reviewer extracts denominator semantics.</t>
+          <t>Keep as context-only unless CDC publishes explicit count/geography data in this source and a reviewer extracts denominator semantics. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -3653,17 +3653,17 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R34"/>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Keep as context-only unless CDC publishes explicit count/geography data in this source and a reviewer extracts denominator semantics.</t>
+          <t>Keep as context-only unless CDC publishes explicit count/geography data in this source and a reviewer extracts denominator semantics. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -28013,7 +28013,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>watch only; not a model input</t>
+          <t>review only; not used in model</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -28033,7 +28033,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Keep the South Kivu/Bukavu item in watch_signals only. Promote to staged_observations and geography inputs only after DRC MoH/INRB, WHO, Africa CDC, or CDC confirms it.</t>
+          <t>Keep the South Kivu/Bukavu item in source-review rows only. Promote to admitted observation rows and geography inputs only after DRC MoH/INRB, WHO, Africa CDC, or CDC confirms it.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">

</xml_diff>

<commit_message>
Prepare May 22 source-review publication surface (#6)
</commit_message>
<xml_diff>
--- a/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
+++ b/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
@@ -2661,7 +2661,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>watch_tier_b_minus</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>claimed_confirmed_fatal_case</t>
+          <t>claimed confirmed fatal case</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2726,17 +2726,17 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>unconfirmed_by_public_health_authority</t>
+          <t>not confirmed by public-health authority</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R25"/>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Promote only if DRC MoH/INRB, WHO, Africa CDC, or CDC publishes South Kivu/Bukavu in confirmed case counts, map, line list, or sitrep with sample date/origin, lab method, health zone, travel history, death status, and epidemiologic link status. An armed-group claim, however widely reported, does not meet this bar on its own.</t>
+          <t>Promote only if DRC MoH/INRB, WHO, Africa CDC, or CDC publishes South Kivu/Bukavu in confirmed case counts, map, line list, or sitrep with sample date/origin, lab method, health zone, travel history, death status, and epidemiologic link status. An armed-group claim, however widely reported, does not meet this bar on its own. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2829,17 +2829,17 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R26"/>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Promote only as policy/travel-monitoring context. Do not promote into case counts, affected-zone geography, or corridor calibration unless CDC publishes count/geography data in the same source.</t>
+          <t>Promote only as policy/travel-monitoring context. Do not promote into case counts, affected-zone geography, or corridor calibration unless CDC publishes count/geography data in the same source. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -2867,7 +2867,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>regional_cross_check_counts_context_only</t>
+          <t>regional cross check counts context only</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2932,17 +2932,17 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R27"/>
@@ -2958,7 +2958,7 @@
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Use ECDC May 21 count values only as cross-check staged observations unless ECDC publishes a primary line-list or explicit correction that supersedes CDC/WHO figures.</t>
+          <t>Use ECDC May 21 count values only as cross-check staged observations unless ECDC publishes a primary line-list or explicit correction that supersedes CDC/WHO figures. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -3035,17 +3035,17 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R28"/>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Promote to staged counts/geography only if the alert contains explicit outbreak figures and a reviewer extracts them with denominator semantics.</t>
+          <t>Promote to staged counts/geography only if the alert contains explicit outbreak figures and a reviewer extracts them with denominator semantics. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -3138,17 +3138,17 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R29"/>
@@ -3164,7 +3164,7 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Keep as readiness context unless WHO AFRO publishes count/geography tables in this source.</t>
+          <t>Keep as readiness context unless WHO AFRO publishes count/geography tables in this source. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3176,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>context_tier_a_minus</t>
+          <t>context tier a minus</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -3241,17 +3241,17 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R30"/>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Keep as response/traveler-monitoring context; do not use as outbreak count input.</t>
+          <t>Keep as response/traveler-monitoring context; do not use as outbreak count input. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>context_tier_b_plus</t>
+          <t>context tier b plus</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3344,17 +3344,17 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>published_context_signal_hash_recorded_bytes</t>
+          <t>published context signal hash recorded bytes</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R31"/>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3427,7 +3427,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>risk_and_response_context</t>
+          <t>risk and response context</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3447,17 +3447,17 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>official_who_statement</t>
+          <t>official who statement</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R32"/>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>Use for risk-context copy and Uganda transmission-status context; do not promote to zone-attributed count input.</t>
+          <t>Use for risk-context copy and Uganda transmission-status context; do not promote to zone-attributed count input. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -3550,17 +3550,17 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R33"/>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>Keep as context-only unless CDC publishes explicit count/geography data in this source and a reviewer extracts denominator semantics.</t>
+          <t>Keep as context-only unless CDC publishes explicit count/geography data in this source and a reviewer extracts denominator semantics. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3588,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>watch_signal</t>
+          <t>source under review</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>context_tier_a</t>
+          <t>context tier a</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>not_a_case_count_source</t>
+          <t>not a case count source</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -3653,17 +3653,17 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>published_context_signal</t>
+          <t>published context signal</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>blocked_pending_official_confirmation</t>
+          <t>not admitted pending official confirmation</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>not_model_input</t>
+          <t>not used in model</t>
         </is>
       </c>
       <c r="R34"/>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Keep as context-only unless CDC publishes explicit count/geography data in this source and a reviewer extracts denominator semantics.</t>
+          <t>Keep as context-only unless CDC publishes explicit count/geography data in this source and a reviewer extracts denominator semantics. Official/public-health promotion gate: do not use for counts, geography, corridor calibration, or model inputs unless an official public-health source publishes explicit count/geography data for that use.</t>
         </is>
       </c>
     </row>
@@ -28013,7 +28013,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>watch only; not a model input</t>
+          <t>review only; not used in model</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -28033,7 +28033,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Keep the South Kivu/Bukavu item in watch_signals only. Promote to staged_observations and geography inputs only after DRC MoH/INRB, WHO, Africa CDC, or CDC confirms it.</t>
+          <t>Keep the South Kivu/Bukavu item in source-review rows only. Promote to admitted observation rows and geography inputs only after DRC MoH/INRB, WHO, Africa CDC, or CDC confirms it.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">

</xml_diff>

<commit_message>
Release LOVS snapshot 2026-05-24 (review-only; not published)
Higher-of-valid-primaries reconciliation: confirmed 88 (CDC 23 May),
suspected 750 (WHO DG 22 May), deaths 177 (WHO DG 22 May). CDC's lower
746 suspected and 176 deaths are retained as dated conflict anchors, not
down-revisions. Corridor watchlist range 0.6-20.7% lower, 1.8-47.0% upper
(suspected feeds the ascertainment denominator). Calibration ledger carried
forward unchanged (12 points, resolves 2026-06-19/20). Regenerated and
verified via release_snapshot.py --check: 263 tests, byte-determinism,
snapshot-contract and evidence-chain gates green.
</commit_message>
<xml_diff>
--- a/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
+++ b/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
@@ -113,7 +113,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-23T23:59:59Z</t>
+          <t>2026-05-24T23:59:59Z</t>
         </is>
       </c>
     </row>
@@ -124,7 +124,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
@@ -2323,8 +2323,66 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Ministere de la Sante Publique, Hygiene et Prevoyance sociale, Democratic Republic of the Congo</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>national_moh</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://administration.sante.gouv.cd/graphql</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-05-24T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-05-24T23:53:59Z</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>f3d5149176d77cbf28d15c79bb7449b1a516c6b855ffe28d51b2adaef0f4bff5</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>private_restricted_bytes</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>publisher-terms-not-confirmed</t>
+        </is>
+      </c>
+      <c r="J37"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L36"/>
+  <autoFilter ref="A1:L37"/>
 </worksheet>
 </file>
 
@@ -4266,7 +4324,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-024</t>
+          <t>BDBV-CLAIM-025</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -4367,7 +4425,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-024</t>
+          <t>BDBV-CLAIM-025</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -4468,7 +4526,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-024</t>
+          <t>BDBV-CLAIM-025</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -9518,12 +9576,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-23T23:59:59Z</t>
+          <t>2026-05-24T23:59:59Z</t>
         </is>
       </c>
       <c r="E2"/>
@@ -9557,7 +9615,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="D3"/>
@@ -14061,8 +14119,129 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>source_data_report_date:drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>source_data_report_date</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="D110"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24</t>
+        </is>
+      </c>
+      <c r="F110"/>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>national_moh</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>recorded</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Data/report date the source says the observation describes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>source_publication_date:drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>source_publication_date</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="D111"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24</t>
+        </is>
+      </c>
+      <c r="F111"/>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>national_moh</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>recorded</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Date the source made the observation available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>source_retrieval_date:drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>source_retrieval_date</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>2026-05-24T23:53:59Z</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24</t>
+        </is>
+      </c>
+      <c r="F112"/>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>national_moh</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>recorded</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Archive capture timestamp for this source edition.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I109"/>
+  <autoFilter ref="A1:I112"/>
 </worksheet>
 </file>
 
@@ -29145,17 +29324,17 @@
       <c r="D191"/>
       <c r="E191" t="inlineStr">
         <is>
-          <t>2026-05-23T23:59:59Z</t>
+          <t>2026-05-24T23:59:59Z</t>
         </is>
       </c>
       <c r="F191">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="G191">
         <v>395</v>
       </c>
       <c r="H191">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="I191" t="inlineStr">
         <is>
@@ -29164,7 +29343,7 @@
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-23</t>
+          <t>who-dg-remarks-bdbv-2026-05-22</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -29189,12 +29368,12 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.who.int/news-room/speeches/item/who-director-general-s-opening-remarks-at-the-member-state-information-session-on-outbreaks-of-ebola-and-hantavirus-22-may-2026</t>
         </is>
       </c>
       <c r="P191" t="inlineStr">
         <is>
-          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
+          <t>40367f2982e766cd8d12f4f223e420d6c4739f4ed1345c8584541619ec061495</t>
         </is>
       </c>
       <c r="Q191" t="inlineStr">
@@ -29204,7 +29383,7 @@
       </c>
       <c r="R191" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-NC-SA-3.0-IGO</t>
         </is>
       </c>
       <c r="S191"/>
@@ -29228,7 +29407,7 @@
       <c r="D192"/>
       <c r="E192" t="inlineStr">
         <is>
-          <t>2026-05-23T23:59:59Z</t>
+          <t>2026-05-24T23:59:59Z</t>
         </is>
       </c>
       <c r="F192">
@@ -29315,11 +29494,11 @@
       <c r="D193"/>
       <c r="E193" t="inlineStr">
         <is>
-          <t>2026-05-23T23:59:59Z</t>
+          <t>2026-05-24T23:59:59Z</t>
         </is>
       </c>
       <c r="F193">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G193">
         <v>106</v>
@@ -29334,7 +29513,7 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-23</t>
+          <t>who-dg-remarks-bdbv-2026-05-22</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -29359,12 +29538,12 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.who.int/news-room/speeches/item/who-director-general-s-opening-remarks-at-the-member-state-information-session-on-outbreaks-of-ebola-and-hantavirus-22-may-2026</t>
         </is>
       </c>
       <c r="P193" t="inlineStr">
         <is>
-          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
+          <t>40367f2982e766cd8d12f4f223e420d6c4739f4ed1345c8584541619ec061495</t>
         </is>
       </c>
       <c r="Q193" t="inlineStr">
@@ -29374,7 +29553,7 @@
       </c>
       <c r="R193" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-NC-SA-3.0-IGO</t>
         </is>
       </c>
       <c r="S193"/>
@@ -40429,7 +40608,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>corridor:01:rwampara:arua-uga</t>
+          <t>corridor:01:rwampara:nebbi-uga</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -40439,33 +40618,33 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D2">
         <v>30</v>
       </c>
       <c r="E2">
-        <v>0.08200892704713533</v>
+        <v>0.08821137528895254</v>
       </c>
       <c r="F2">
-        <v>0.23133172037904387</v>
+        <v>0.22303064012958748</v>
       </c>
       <c r="G2">
-        <v>0.19224680649154585</v>
+        <v>0.20708736075627046</v>
       </c>
       <c r="H2">
-        <v>0.48130923946896836</v>
+        <v>0.46958460345401354</v>
       </c>
       <c r="I2">
-        <v>0.053772224744336926</v>
+        <v>0.04902386658584786</v>
       </c>
       <c r="J2">
-        <v>0.7505179739127573</v>
+        <v>0.7287947804941787</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -40497,7 +40676,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>corridor:02:rwampara:nebbi-uga</t>
+          <t>corridor:02:rwampara:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -40507,33 +40686,33 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D3">
         <v>30</v>
       </c>
       <c r="E3">
-        <v>0.09073176115266587</v>
+        <v>0.08379468993464778</v>
       </c>
       <c r="F3">
-        <v>0.2234638809118071</v>
+        <v>0.21991047250618512</v>
       </c>
       <c r="G3">
-        <v>0.2112617269468639</v>
+        <v>0.1974008464379203</v>
       </c>
       <c r="H3">
-        <v>0.4679601163839139</v>
+        <v>0.4642163934402524</v>
       </c>
       <c r="I3">
-        <v>0.05444279683836906</v>
+        <v>0.053885607469128294</v>
       </c>
       <c r="J3">
-        <v>0.7258589806643395</v>
+        <v>0.7321362714426363</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -40565,7 +40744,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>corridor:03:rwampara:bundibugyo-uga</t>
+          <t>corridor:03:rwampara:arua-uga</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -40575,33 +40754,33 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D4">
         <v>30</v>
       </c>
       <c r="E4">
-        <v>0.08561119889466778</v>
+        <v>0.0839815096390503</v>
       </c>
       <c r="F4">
-        <v>0.22176004554817166</v>
+        <v>0.2145009745062685</v>
       </c>
       <c r="G4">
-        <v>0.20013232620824334</v>
+        <v>0.1978119698305737</v>
       </c>
       <c r="H4">
-        <v>0.46504340386236126</v>
+        <v>0.4548317738545009</v>
       </c>
       <c r="I4">
-        <v>0.047305248394329626</v>
+        <v>0.05127631522501777</v>
       </c>
       <c r="J4">
-        <v>0.7273888815013723</v>
+        <v>0.7081902165953425</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -40633,7 +40812,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>corridor:04:rwampara:beni-cod</t>
+          <t>corridor:04:rwampara:kampala-uga</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -40643,33 +40822,33 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D5">
         <v>30</v>
       </c>
       <c r="E5">
-        <v>0.08965956893852142</v>
+        <v>0.08494514057794225</v>
       </c>
       <c r="F5">
-        <v>0.22137061515466477</v>
+        <v>0.21235423218408028</v>
       </c>
       <c r="G5">
-        <v>0.20893910254125775</v>
+        <v>0.1999306534527504</v>
       </c>
       <c r="H5">
-        <v>0.46437526414832964</v>
+        <v>0.4510801786497356</v>
       </c>
       <c r="I5">
-        <v>0.052399160989858806</v>
+        <v>0.05148499356098289</v>
       </c>
       <c r="J5">
-        <v>0.7341199202505713</v>
+        <v>0.7157785863906272</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -40701,7 +40880,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>corridor:05:rwampara:kampala-uga</t>
+          <t>corridor:05:rwampara:beni-cod</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -40711,33 +40890,33 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D6">
         <v>30</v>
       </c>
       <c r="E6">
-        <v>0.07930621278103206</v>
+        <v>0.08478074397061586</v>
       </c>
       <c r="F6">
-        <v>0.21778218088702597</v>
+        <v>0.207375477491343</v>
       </c>
       <c r="G6">
-        <v>0.1862999889886741</v>
+        <v>0.19956967743719028</v>
       </c>
       <c r="H6">
-        <v>0.4581946240505208</v>
+        <v>0.44231999358257157</v>
       </c>
       <c r="I6">
-        <v>0.04942555665634105</v>
+        <v>0.06353899831251818</v>
       </c>
       <c r="J6">
-        <v>0.6940368144191931</v>
+        <v>0.7043971359810433</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -40786,26 +40965,26 @@
         <v>30</v>
       </c>
       <c r="E7">
-        <v>0.08030398782374049</v>
+        <v>0.08325361349716673</v>
       </c>
       <c r="F7">
-        <v>0.21293669407875018</v>
+        <v>0.1998336728649868</v>
       </c>
       <c r="G7">
-        <v>0.1884976810866289</v>
+        <v>0.19620947023756097</v>
       </c>
       <c r="H7">
-        <v>0.44978058214750455</v>
+        <v>0.42888994329056224</v>
       </c>
       <c r="I7">
-        <v>0.05948655613109171</v>
+        <v>0.06493900025049605</v>
       </c>
       <c r="J7">
-        <v>0.7008370348305115</v>
+        <v>0.6577801207519675</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 31 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -40837,7 +41016,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>corridor:07:bunia:arua-uga</t>
+          <t>corridor:07:bunia:nebbi-uga</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -40847,33 +41026,33 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D8">
         <v>30</v>
       </c>
       <c r="E8">
-        <v>0.043126410860172215</v>
+        <v>0.04518668590906155</v>
       </c>
       <c r="F8">
-        <v>0.1223867538035171</v>
+        <v>0.1196025189042455</v>
       </c>
       <c r="G8">
-        <v>0.10415994692106009</v>
+        <v>0.10969096522136429</v>
       </c>
       <c r="H8">
-        <v>0.278001397537348</v>
+        <v>0.27390511702374754</v>
       </c>
       <c r="I8">
-        <v>0.02384393205347049</v>
+        <v>0.028519411921781153</v>
       </c>
       <c r="J8">
-        <v>0.4522298484507357</v>
+        <v>0.47620777811346965</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -40905,7 +41084,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>corridor:08:bunia:kasese-uga</t>
+          <t>corridor:08:bunia:beni-cod</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -40915,33 +41094,33 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D9">
         <v>30</v>
       </c>
       <c r="E9">
-        <v>0.03942345667630251</v>
+        <v>0.04272194828018169</v>
       </c>
       <c r="F9">
-        <v>0.11196397554917834</v>
+        <v>0.11698145631419321</v>
       </c>
       <c r="G9">
-        <v>0.09548507505855064</v>
+        <v>0.10390491590127435</v>
       </c>
       <c r="H9">
-        <v>0.25641649420715795</v>
+        <v>0.26846117499318517</v>
       </c>
       <c r="I9">
-        <v>0.02390916867239624</v>
+        <v>0.036396743130945</v>
       </c>
       <c r="J9">
-        <v>0.44162866614763796</v>
+        <v>0.48307011246840226</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -40973,12 +41152,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>corridor:09:bunia:kampala-uga</t>
+          <t>corridor:09:mongbwalu:kampala-uga</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>bunia</t>
+          <t>mongbwalu</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -40990,26 +41169,26 @@
         <v>30</v>
       </c>
       <c r="E10">
-        <v>0.04202315052143141</v>
+        <v>0.04490334467385315</v>
       </c>
       <c r="F10">
-        <v>0.11138026974825257</v>
+        <v>0.11650060274026874</v>
       </c>
       <c r="G10">
-        <v>0.10158065236044309</v>
+        <v>0.10902687738091718</v>
       </c>
       <c r="H10">
-        <v>0.2551963318474184</v>
+        <v>0.2674597792030441</v>
       </c>
       <c r="I10">
-        <v>0.028293248051654254</v>
+        <v>0.028105747197389272</v>
       </c>
       <c r="J10">
-        <v>0.47040250224193386</v>
+        <v>0.48254317209197545</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -41041,7 +41220,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>corridor:10:bunia:beni-cod</t>
+          <t>corridor:10:bunia:arua-uga</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -41051,33 +41230,33 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D11">
         <v>30</v>
       </c>
       <c r="E11">
-        <v>0.03846581360295262</v>
+        <v>0.04266596415746421</v>
       </c>
       <c r="F11">
-        <v>0.10908382568535815</v>
+        <v>0.11566773655391216</v>
       </c>
       <c r="G11">
-        <v>0.09323346947609981</v>
+        <v>0.103773243645609</v>
       </c>
       <c r="H11">
-        <v>0.250384634775751</v>
+        <v>0.26572331467385835</v>
       </c>
       <c r="I11">
-        <v>0.026991287216266743</v>
+        <v>0.030154900882461463</v>
       </c>
       <c r="J11">
-        <v>0.44466813809985917</v>
+        <v>0.47857090928303725</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -41109,43 +41288,43 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>corridor:11:mongbwalu:bundibugyo-uga</t>
+          <t>corridor:11:bunia:kasese-uga</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>mongbwalu</t>
+          <t>bunia</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D12">
         <v>30</v>
       </c>
       <c r="E12">
-        <v>0.04041524745754471</v>
+        <v>0.04134626185720458</v>
       </c>
       <c r="F12">
-        <v>0.10894918908127146</v>
+        <v>0.11536982131263696</v>
       </c>
       <c r="G12">
-        <v>0.09781348907649148</v>
+        <v>0.1006654147151124</v>
       </c>
       <c r="H12">
-        <v>0.2501020107590719</v>
+        <v>0.2651016560931514</v>
       </c>
       <c r="I12">
-        <v>0.024679096234898047</v>
+        <v>0.024157414736271563</v>
       </c>
       <c r="J12">
-        <v>0.46678405365895886</v>
+        <v>0.442217743189379</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -41177,43 +41356,43 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>corridor:12:bunia:bundibugyo-uga</t>
+          <t>corridor:12:mongbwalu:nebbi-uga</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>bunia</t>
+          <t>mongbwalu</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D13">
         <v>30</v>
       </c>
       <c r="E13">
-        <v>0.04019611700549866</v>
+        <v>0.042257015039710716</v>
       </c>
       <c r="F13">
-        <v>0.10812598156102118</v>
+        <v>0.11059749483342382</v>
       </c>
       <c r="G13">
-        <v>0.09729907368089252</v>
+        <v>0.1028109484353942</v>
       </c>
       <c r="H13">
-        <v>0.24837217550661125</v>
+        <v>0.25509913387234384</v>
       </c>
       <c r="I13">
-        <v>0.01923753856147162</v>
+        <v>0.029949093157880583</v>
       </c>
       <c r="J13">
-        <v>0.44227089655366103</v>
+        <v>0.44975839331305956</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -41245,7 +41424,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>corridor:13:mongbwalu:beni-cod</t>
+          <t>corridor:13:mongbwalu:kasese-uga</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -41255,33 +41434,33 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D14">
         <v>30</v>
       </c>
       <c r="E14">
-        <v>0.040819990834027126</v>
+        <v>0.036835801322681855</v>
       </c>
       <c r="F14">
-        <v>0.10618433430550114</v>
+        <v>0.1084031822966573</v>
       </c>
       <c r="G14">
-        <v>0.09876265362816536</v>
+        <v>0.08999553522869064</v>
       </c>
       <c r="H14">
-        <v>0.2442825392959079</v>
+        <v>0.250472627736926</v>
       </c>
       <c r="I14">
-        <v>0.020678655931406387</v>
+        <v>0.027203361343210414</v>
       </c>
       <c r="J14">
-        <v>0.4596848493726443</v>
+        <v>0.4354015904706045</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -41313,7 +41492,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>corridor:14:bunia:nebbi-uga</t>
+          <t>corridor:14:bunia:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -41323,33 +41502,33 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D15">
         <v>30</v>
       </c>
       <c r="E15">
-        <v>0.04472132043254323</v>
+        <v>0.04255734933972799</v>
       </c>
       <c r="F15">
-        <v>0.10504297781519889</v>
+        <v>0.10802646318829781</v>
       </c>
       <c r="G15">
-        <v>0.10788098545533736</v>
+        <v>0.10351772313795171</v>
       </c>
       <c r="H15">
-        <v>0.24187270316516957</v>
+        <v>0.24967485196493885</v>
       </c>
       <c r="I15">
-        <v>0.02260695551444377</v>
+        <v>0.02764874782267757</v>
       </c>
       <c r="J15">
-        <v>0.4282924026162399</v>
+        <v>0.446580559517115</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -41381,12 +41560,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>corridor:15:mongbwalu:kampala-uga</t>
+          <t>corridor:15:bunia:kampala-uga</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>mongbwalu</t>
+          <t>bunia</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -41398,26 +41577,26 @@
         <v>30</v>
       </c>
       <c r="E16">
-        <v>0.03779941060386105</v>
+        <v>0.03947505835897319</v>
       </c>
       <c r="F16">
-        <v>0.10451891208285768</v>
+        <v>0.10766293076106442</v>
       </c>
       <c r="G16">
-        <v>0.09166463393260285</v>
+        <v>0.09624824633100992</v>
       </c>
       <c r="H16">
-        <v>0.2407645390707007</v>
+        <v>0.24890792140087264</v>
       </c>
       <c r="I16">
-        <v>0.027657720160362238</v>
+        <v>0.023441943477585433</v>
       </c>
       <c r="J16">
-        <v>0.4396111744978209</v>
+        <v>0.4469881708758133</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -41449,7 +41628,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>corridor:16:mongbwalu:kasese-uga</t>
+          <t>corridor:16:mongbwalu:arua-uga</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -41459,33 +41638,33 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D17">
         <v>30</v>
       </c>
       <c r="E17">
-        <v>0.04170004663803706</v>
+        <v>0.037054326822585304</v>
       </c>
       <c r="F17">
-        <v>0.10372098668085056</v>
+        <v>0.10690154315918662</v>
       </c>
       <c r="G17">
-        <v>0.1008243915792412</v>
+        <v>0.09051412784116997</v>
       </c>
       <c r="H17">
-        <v>0.2390754226533218</v>
+        <v>0.24729635769244965</v>
       </c>
       <c r="I17">
-        <v>0.028925700788658745</v>
+        <v>0.023841914883054538</v>
       </c>
       <c r="J17">
-        <v>0.4110297404446275</v>
+        <v>0.41691596849067886</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -41517,7 +41696,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>corridor:17:mongbwalu:arua-uga</t>
+          <t>corridor:17:mongbwalu:beni-cod</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -41527,33 +41706,33 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D18">
         <v>30</v>
       </c>
       <c r="E18">
-        <v>0.035186585343488896</v>
+        <v>0.03751084235818841</v>
       </c>
       <c r="F18">
-        <v>0.1022202018711377</v>
+        <v>0.10663402594128604</v>
       </c>
       <c r="G18">
-        <v>0.08549785806756499</v>
+        <v>0.09159725797748078</v>
       </c>
       <c r="H18">
-        <v>0.23589234541472318</v>
+        <v>0.24672965162274357</v>
       </c>
       <c r="I18">
-        <v>0.027502933564814515</v>
+        <v>0.02407954679637498</v>
       </c>
       <c r="J18">
-        <v>0.40677152882419465</v>
+        <v>0.44454587739519735</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -41585,7 +41764,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>corridor:18:mongbwalu:nebbi-uga</t>
+          <t>corridor:18:mongbwalu:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -41595,33 +41774,33 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D19">
         <v>30</v>
       </c>
       <c r="E19">
-        <v>0.03874391914011116</v>
+        <v>0.040216833909035604</v>
       </c>
       <c r="F19">
-        <v>0.09932753400748234</v>
+        <v>0.10227893881178257</v>
       </c>
       <c r="G19">
-        <v>0.0938876818934965</v>
+        <v>0.09800089155866029</v>
       </c>
       <c r="H19">
-        <v>0.22973469142772449</v>
+        <v>0.23746750551426188</v>
       </c>
       <c r="I19">
-        <v>0.02713466345582947</v>
+        <v>0.02574109924333239</v>
       </c>
       <c r="J19">
-        <v>0.43207387785922474</v>
+        <v>0.4462240901573336</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -41653,7 +41832,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>corridor:19:nyankunde:kasese-uga</t>
+          <t>corridor:19:nyankunde:nebbi-uga</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -41663,33 +41842,33 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D20">
         <v>30</v>
       </c>
       <c r="E20">
-        <v>0.03299388535147604</v>
+        <v>0.03239630370940688</v>
       </c>
       <c r="F20">
-        <v>0.08738286997481087</v>
+        <v>0.09379632815128686</v>
       </c>
       <c r="G20">
-        <v>0.08030326285925304</v>
+        <v>0.07941922175273045</v>
       </c>
       <c r="H20">
-        <v>0.2039935043660834</v>
+        <v>0.21923462953102077</v>
       </c>
       <c r="I20">
-        <v>0.019930168144148393</v>
+        <v>0.020658583016893068</v>
       </c>
       <c r="J20">
-        <v>0.3775284009544754</v>
+        <v>0.3757448935253982</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -41721,7 +41900,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>corridor:20:nyankunde:beni-cod</t>
+          <t>corridor:20:nyankunde:kampala-uga</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -41731,33 +41910,33 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D21">
         <v>30</v>
       </c>
       <c r="E21">
-        <v>0.03392819706306785</v>
+        <v>0.031343249954173036</v>
       </c>
       <c r="F21">
-        <v>0.08484940586882139</v>
+        <v>0.08962807165406164</v>
       </c>
       <c r="G21">
-        <v>0.0825188916401238</v>
+        <v>0.07689972645270565</v>
       </c>
       <c r="H21">
-        <v>0.19846854926794583</v>
+        <v>0.21017937050599006</v>
       </c>
       <c r="I21">
-        <v>0.024490234067551103</v>
+        <v>0.020495136113379064</v>
       </c>
       <c r="J21">
-        <v>0.37749315707435055</v>
+        <v>0.3809572978186992</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -41789,7 +41968,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>corridor:21:nyankunde:nebbi-uga</t>
+          <t>corridor:21:nyankunde:arua-uga</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -41799,33 +41978,33 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D22">
         <v>30</v>
       </c>
       <c r="E22">
-        <v>0.03125577174100408</v>
+        <v>0.03310879855573873</v>
       </c>
       <c r="F22">
-        <v>0.08348454522926196</v>
+        <v>0.08657015317950179</v>
       </c>
       <c r="G22">
-        <v>0.0761732305165149</v>
+        <v>0.08112150891437181</v>
       </c>
       <c r="H22">
-        <v>0.19548267507850767</v>
+        <v>0.20349621355211361</v>
       </c>
       <c r="I22">
-        <v>0.02440925206055355</v>
+        <v>0.02417182913316858</v>
       </c>
       <c r="J22">
-        <v>0.37594067840426554</v>
+        <v>0.3559785151431059</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -41857,7 +42036,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>corridor:22:nyankunde:kampala-uga</t>
+          <t>corridor:22:nyankunde:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -41867,33 +42046,33 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D23">
         <v>30</v>
       </c>
       <c r="E23">
-        <v>0.031478646822295314</v>
+        <v>0.027757679481219877</v>
       </c>
       <c r="F23">
-        <v>0.08284362872862142</v>
+        <v>0.08316271163642758</v>
       </c>
       <c r="G23">
-        <v>0.07670344805404702</v>
+        <v>0.06828987627797062</v>
       </c>
       <c r="H23">
-        <v>0.1940782082884187</v>
+        <v>0.19600919074702933</v>
       </c>
       <c r="I23">
-        <v>0.02186039936076743</v>
+        <v>0.01652290575782679</v>
       </c>
       <c r="J23">
-        <v>0.36475291410219285</v>
+        <v>0.35346265816565353</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -41925,7 +42104,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>corridor:23:nyankunde:arua-uga</t>
+          <t>corridor:23:nyankunde:kasese-uga</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -41935,33 +42114,33 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D24">
         <v>30</v>
       </c>
       <c r="E24">
-        <v>0.029994277699168237</v>
+        <v>0.029262518404558985</v>
       </c>
       <c r="F24">
-        <v>0.0826132813539486</v>
+        <v>0.0827973940167662</v>
       </c>
       <c r="G24">
-        <v>0.07316870543259008</v>
+        <v>0.0719092309443406</v>
       </c>
       <c r="H24">
-        <v>0.19357307850580524</v>
+        <v>0.19520396884789892</v>
       </c>
       <c r="I24">
-        <v>0.016047833475468353</v>
+        <v>0.0160365093845038</v>
       </c>
       <c r="J24">
-        <v>0.3573780111640004</v>
+        <v>0.37244943158791305</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -41993,7 +42172,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>corridor:24:nyankunde:bundibugyo-uga</t>
+          <t>corridor:24:nyankunde:beni-cod</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -42003,33 +42182,33 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D25">
         <v>30</v>
       </c>
       <c r="E25">
-        <v>0.028661907391696856</v>
+        <v>0.029014915856687168</v>
       </c>
       <c r="F25">
-        <v>0.08085785766740855</v>
+        <v>0.07992581840442112</v>
       </c>
       <c r="G25">
-        <v>0.06998902920795538</v>
+        <v>0.07131428938994647</v>
       </c>
       <c r="H25">
-        <v>0.18971739841881297</v>
+        <v>0.18885779917755408</v>
       </c>
       <c r="I25">
-        <v>0.018016370547401035</v>
+        <v>0.026204983312365895</v>
       </c>
       <c r="J25">
-        <v>0.36065493954245237</v>
+        <v>0.39197883927654326</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 11 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -42061,7 +42240,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>corridor:25:katwa:bundibugyo-uga</t>
+          <t>corridor:25:katwa:arua-uga</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -42071,33 +42250,33 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D26">
         <v>30</v>
       </c>
       <c r="E26">
-        <v>0.005793429794588911</v>
+        <v>0.006120542874036516</v>
       </c>
       <c r="F26">
-        <v>0.01702984566490226</v>
+        <v>0.01699417338751852</v>
       </c>
       <c r="G26">
-        <v>0.01439258175594163</v>
+        <v>0.015308080460276235</v>
       </c>
       <c r="H26">
-        <v>0.041951574982737355</v>
+        <v>0.042154297513636585</v>
       </c>
       <c r="I26">
-        <v>0.0038181048856288867</v>
+        <v>0.003537521039203559</v>
       </c>
       <c r="J26">
-        <v>0.08616420003025087</v>
+        <v>0.08297678927478849</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -42129,7 +42308,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>corridor:26:katwa:beni-cod</t>
+          <t>corridor:26:katwa:kasese-uga</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -42139,33 +42318,33 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D27">
         <v>30</v>
       </c>
       <c r="E27">
-        <v>0.005897051963327515</v>
+        <v>0.005874612094265597</v>
       </c>
       <c r="F27">
-        <v>0.016454298957175345</v>
+        <v>0.016526384306946418</v>
       </c>
       <c r="G27">
-        <v>0.01464887215333438</v>
+        <v>0.014695723098220564</v>
       </c>
       <c r="H27">
-        <v>0.04055132576639631</v>
+        <v>0.041008547755741837</v>
       </c>
       <c r="I27">
-        <v>0.0035690102911354387</v>
+        <v>0.0034953489095219947</v>
       </c>
       <c r="J27">
-        <v>0.08080632138202076</v>
+        <v>0.07196869182617144</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -42197,7 +42376,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>corridor:27:katwa:nebbi-uga</t>
+          <t>corridor:27:katwa:kampala-uga</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -42207,33 +42386,33 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D28">
         <v>30</v>
       </c>
       <c r="E28">
-        <v>0.006239312368845673</v>
+        <v>0.0063472860999863046</v>
       </c>
       <c r="F28">
-        <v>0.01619803151236343</v>
+        <v>0.016310473511373214</v>
       </c>
       <c r="G28">
-        <v>0.015495105961945144</v>
+        <v>0.015872457611902313</v>
       </c>
       <c r="H28">
-        <v>0.039927464536473806</v>
+        <v>0.0404794429759861</v>
       </c>
       <c r="I28">
-        <v>0.003405178314087784</v>
+        <v>0.0036262347035018044</v>
       </c>
       <c r="J28">
-        <v>0.07935673326585045</v>
+        <v>0.08668303567476036</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -42265,7 +42444,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>corridor:28:katwa:kampala-uga</t>
+          <t>corridor:28:katwa:beni-cod</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -42275,33 +42454,33 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D29">
         <v>30</v>
       </c>
       <c r="E29">
-        <v>0.006392865452645141</v>
+        <v>0.005674021075253249</v>
       </c>
       <c r="F29">
-        <v>0.016120155850815304</v>
+        <v>0.015966822911828493</v>
       </c>
       <c r="G29">
-        <v>0.01587462279882418</v>
+        <v>0.014196090807731543</v>
       </c>
       <c r="H29">
-        <v>0.03973783345894116</v>
+        <v>0.039636938611780054</v>
       </c>
       <c r="I29">
-        <v>0.0032650126802971193</v>
+        <v>0.0034806849422171797</v>
       </c>
       <c r="J29">
-        <v>0.07658764416722781</v>
+        <v>0.0780554614612525</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -42333,7 +42512,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>corridor:29:katwa:kasese-uga</t>
+          <t>corridor:29:katwa:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -42343,33 +42522,33 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D30">
         <v>30</v>
       </c>
       <c r="E30">
-        <v>0.005897977372847696</v>
+        <v>0.0064256354798581106</v>
       </c>
       <c r="F30">
-        <v>0.016114027975795253</v>
+        <v>0.015695763569745308</v>
       </c>
       <c r="G30">
-        <v>0.014651160795670248</v>
+        <v>0.016067429277709516</v>
       </c>
       <c r="H30">
-        <v>0.039722906756456705</v>
+        <v>0.038972088119423404</v>
       </c>
       <c r="I30">
-        <v>0.004563029278651646</v>
+        <v>0.00498049465626442</v>
       </c>
       <c r="J30">
-        <v>0.08758262782791992</v>
+        <v>0.0758544841015686</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -42401,7 +42580,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>corridor:30:katwa:arua-uga</t>
+          <t>corridor:30:katwa:nebbi-uga</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -42411,33 +42590,33 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D31">
         <v>30</v>
       </c>
       <c r="E31">
-        <v>0.0053809689229898094</v>
+        <v>0.005382307947903675</v>
       </c>
       <c r="F31">
-        <v>0.014969127663845894</v>
+        <v>0.015689028622659945</v>
       </c>
       <c r="G31">
-        <v>0.013372039811872988</v>
+        <v>0.013469218884625184</v>
       </c>
       <c r="H31">
-        <v>0.036932402731466474</v>
+        <v>0.038955562840755714</v>
       </c>
       <c r="I31">
-        <v>0.0043470653458970695</v>
+        <v>0.00261336226616051</v>
       </c>
       <c r="J31">
-        <v>0.0819411234458965</v>
+        <v>0.08089104819780216</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 2 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -42469,12 +42648,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>corridor:31:miti-murhesa:nebbi-uga</t>
+          <t>corridor:31:nizi:nebbi-uga</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>miti-murhesa</t>
+          <t>nizi</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -42486,26 +42665,26 @@
         <v>30</v>
       </c>
       <c r="E32">
-        <v>0.0031064099748497886</v>
+        <v>0.003036170632948393</v>
       </c>
       <c r="F32">
-        <v>0.008842744721272167</v>
+        <v>0.008699255524416832</v>
       </c>
       <c r="G32">
-        <v>0.00773278016050985</v>
+        <v>0.007611531620020595</v>
       </c>
       <c r="H32">
-        <v>0.021917803930031482</v>
+        <v>0.02171516880923019</v>
       </c>
       <c r="I32">
-        <v>0.0012927920382234503</v>
+        <v>0.0018231578456973485</v>
       </c>
       <c r="J32">
-        <v>0.043151428768583286</v>
+        <v>0.0406946321513916</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -42537,12 +42716,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>corridor:32:nizi:kasese-uga</t>
+          <t>corridor:32:miti-murhesa:kasese-uga</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>nizi</t>
+          <t>miti-murhesa</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -42554,26 +42733,26 @@
         <v>30</v>
       </c>
       <c r="E33">
-        <v>0.0030137247816908463</v>
+        <v>0.003044055247326788</v>
       </c>
       <c r="F33">
-        <v>0.008455401394654921</v>
+        <v>0.00860046134544773</v>
       </c>
       <c r="G33">
-        <v>0.007502579723034392</v>
+        <v>0.007631252063973859</v>
       </c>
       <c r="H33">
-        <v>0.020963818333134487</v>
+        <v>0.021470167816893482</v>
       </c>
       <c r="I33">
-        <v>0.001964876026614837</v>
+        <v>0.0014973330122456524</v>
       </c>
       <c r="J33">
-        <v>0.04025996291249157</v>
+        <v>0.038352523140163956</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -42605,43 +42784,43 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>corridor:33:bambu:kasese-uga</t>
+          <t>corridor:33:miti-murhesa:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>miti-murhesa</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D34">
         <v>30</v>
       </c>
       <c r="E34">
-        <v>0.0028886304443923594</v>
+        <v>0.002981208606110952</v>
       </c>
       <c r="F34">
-        <v>0.008347118481784016</v>
+        <v>0.00853010671090837</v>
       </c>
       <c r="G34">
-        <v>0.00719183460774292</v>
+        <v>0.007474055522301043</v>
       </c>
       <c r="H34">
-        <v>0.020697029082573037</v>
+        <v>0.021295671112063014</v>
       </c>
       <c r="I34">
-        <v>0.0017626325075392108</v>
+        <v>0.0020763684021678276</v>
       </c>
       <c r="J34">
-        <v>0.040846686395662496</v>
+        <v>0.04157524175982064</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -42673,43 +42852,43 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>corridor:34:nizi:bundibugyo-uga</t>
+          <t>corridor:34:butembo:nebbi-uga</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>nizi</t>
+          <t>butembo</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D35">
         <v>30</v>
       </c>
       <c r="E35">
-        <v>0.003021126031914151</v>
+        <v>0.003049904014779198</v>
       </c>
       <c r="F35">
-        <v>0.008312163807679601</v>
+        <v>0.008510247131509524</v>
       </c>
       <c r="G35">
-        <v>0.0075209637361464965</v>
+        <v>0.0076458810373161434</v>
       </c>
       <c r="H35">
-        <v>0.02061089733019217</v>
+        <v>0.02124641212086062</v>
       </c>
       <c r="I35">
-        <v>0.001965199157311942</v>
+        <v>0.001894892164408163</v>
       </c>
       <c r="J35">
-        <v>0.04232624078531671</v>
+        <v>0.03868551246151107</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -42741,43 +42920,43 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>corridor:35:goma-cod:beni-cod</t>
+          <t>corridor:35:butembo:kasese-uga</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>butembo</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D36">
         <v>30</v>
       </c>
       <c r="E36">
-        <v>0.0029885689228487944</v>
+        <v>0.00310326252679316</v>
       </c>
       <c r="F36">
-        <v>0.008309165031427646</v>
+        <v>0.008371286435940095</v>
       </c>
       <c r="G36">
-        <v>0.0074400943892386495</v>
+        <v>0.007779332263353617</v>
       </c>
       <c r="H36">
-        <v>0.020603508791962988</v>
+        <v>0.020901691773522968</v>
       </c>
       <c r="I36">
-        <v>0.0015140627043773254</v>
+        <v>0.0017729400819647607</v>
       </c>
       <c r="J36">
-        <v>0.039636236358234156</v>
+        <v>0.041854022880361594</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -42809,43 +42988,43 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>corridor:36:kilo:kampala-uga</t>
+          <t>corridor:36:bambu:arua-uga</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>kilo</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D37">
         <v>30</v>
       </c>
       <c r="E37">
-        <v>0.0028968958480735663</v>
+        <v>0.002967388107118135</v>
       </c>
       <c r="F37">
-        <v>0.008302699189387669</v>
+        <v>0.008337126650148213</v>
       </c>
       <c r="G37">
-        <v>0.007212368681008802</v>
+        <v>0.007439484701364463</v>
       </c>
       <c r="H37">
-        <v>0.02058757493019797</v>
+        <v>0.02081694028687528</v>
       </c>
       <c r="I37">
-        <v>0.0014728301522307502</v>
+        <v>0.0017431353970841308</v>
       </c>
       <c r="J37">
-        <v>0.040142399138471466</v>
+        <v>0.03987425157869348</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -42877,43 +43056,43 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>corridor:37:miti-murhesa:beni-cod</t>
+          <t>corridor:37:butembo:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>miti-murhesa</t>
+          <t>butembo</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D38">
         <v>30</v>
       </c>
       <c r="E38">
-        <v>0.0027436360542250626</v>
+        <v>0.0028635878048932917</v>
       </c>
       <c r="F38">
-        <v>0.008291615601552393</v>
+        <v>0.0083314394748491</v>
       </c>
       <c r="G38">
-        <v>0.006831583025491139</v>
+        <v>0.007179812848703837</v>
       </c>
       <c r="H38">
-        <v>0.020560263716459554</v>
+        <v>0.020802829539148276</v>
       </c>
       <c r="I38">
-        <v>0.001809788062056189</v>
+        <v>0.00148959781119683</v>
       </c>
       <c r="J38">
-        <v>0.04035120838517614</v>
+        <v>0.04118234481782838</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -42945,12 +43124,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>corridor:38:bambu:kampala-uga</t>
+          <t>corridor:38:nizi:kampala-uga</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>nizi</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -42962,26 +43141,26 @@
         <v>30</v>
       </c>
       <c r="E39">
-        <v>0.0028878037106492283</v>
+        <v>0.0028297038262589114</v>
       </c>
       <c r="F39">
-        <v>0.00826700300096575</v>
+        <v>0.008276409421757808</v>
       </c>
       <c r="G39">
-        <v>0.00718978103506368</v>
+        <v>0.0070950385508476155</v>
       </c>
       <c r="H39">
-        <v>0.0204996068255012</v>
+        <v>0.020666287769637415</v>
       </c>
       <c r="I39">
-        <v>0.0015583380599284798</v>
+        <v>0.0016817624400032954</v>
       </c>
       <c r="J39">
-        <v>0.04029488629595264</v>
+        <v>0.039287175973469944</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -43013,12 +43192,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>corridor:39:nizi:kampala-uga</t>
+          <t>corridor:39:goma-cod:kampala-uga</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>nizi</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -43030,26 +43209,26 @@
         <v>30</v>
       </c>
       <c r="E40">
-        <v>0.0030739891390453022</v>
+        <v>0.0028541855896696833</v>
       </c>
       <c r="F40">
-        <v>0.008190495185341068</v>
+        <v>0.008252562887683529</v>
       </c>
       <c r="G40">
-        <v>0.00765226137795097</v>
+        <v>0.007156290108511709</v>
       </c>
       <c r="H40">
-        <v>0.020311061195146723</v>
+        <v>0.020607115412800053</v>
       </c>
       <c r="I40">
-        <v>0.0019126404305481878</v>
+        <v>0.0018998622437845641</v>
       </c>
       <c r="J40">
-        <v>0.03892464933729348</v>
+        <v>0.044504858617887194</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -43081,7 +43260,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>corridor:40:miti-murhesa:bundibugyo-uga</t>
+          <t>corridor:40:miti-murhesa:arua-uga</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -43091,33 +43270,33 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D41">
         <v>30</v>
       </c>
       <c r="E41">
-        <v>0.0030168065956937273</v>
+        <v>0.0027349409401292712</v>
       </c>
       <c r="F41">
-        <v>0.008186419166028969</v>
+        <v>0.008245046196641154</v>
       </c>
       <c r="G41">
-        <v>0.0075102348731063695</v>
+        <v>0.006857927560041555</v>
       </c>
       <c r="H41">
-        <v>0.02030101473563603</v>
+        <v>0.02058846320226515</v>
       </c>
       <c r="I41">
-        <v>0.0019468904654919932</v>
+        <v>0.0014529959377463596</v>
       </c>
       <c r="J41">
-        <v>0.040363293600190024</v>
+        <v>0.03976609261069776</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -43149,43 +43328,43 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>corridor:41:bambu:arua-uga</t>
+          <t>corridor:41:nizi:kasese-uga</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>nizi</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D42">
         <v>30</v>
       </c>
       <c r="E42">
-        <v>0.002768603266617875</v>
+        <v>0.0027780375306676874</v>
       </c>
       <c r="F42">
-        <v>0.008162493230156248</v>
+        <v>0.008203146144269508</v>
       </c>
       <c r="G42">
-        <v>0.006893621987128173</v>
+        <v>0.006965766035151089</v>
       </c>
       <c r="H42">
-        <v>0.020242046539878572</v>
+        <v>0.0204844874721663</v>
       </c>
       <c r="I42">
-        <v>0.0015474160854732802</v>
+        <v>0.001978216297492336</v>
       </c>
       <c r="J42">
-        <v>0.03915694943543016</v>
+        <v>0.03713845609642502</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -43217,7 +43396,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>corridor:42:nizi:nebbi-uga</t>
+          <t>corridor:42:nizi:arua-uga</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -43227,33 +43406,33 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D43">
         <v>30</v>
       </c>
       <c r="E43">
-        <v>0.0029572181128099673</v>
+        <v>0.0029523334159434755</v>
       </c>
       <c r="F43">
-        <v>0.008136926158356317</v>
+        <v>0.008135009614384153</v>
       </c>
       <c r="G43">
-        <v>0.007362219916885793</v>
+        <v>0.007401825721503413</v>
       </c>
       <c r="H43">
-        <v>0.02017903013560457</v>
+        <v>0.02031539108547792</v>
       </c>
       <c r="I43">
-        <v>0.0014210452648333984</v>
+        <v>0.0018778692608227316</v>
       </c>
       <c r="J43">
-        <v>0.03953044137015703</v>
+        <v>0.04145132009147697</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -43285,43 +43464,43 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>corridor:43:butembo:arua-uga</t>
+          <t>corridor:43:goma-cod:beni-cod</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>butembo</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D44">
         <v>30</v>
       </c>
       <c r="E44">
-        <v>0.0028588847097371084</v>
+        <v>0.0030619690333943683</v>
       </c>
       <c r="F44">
-        <v>0.008121479547922666</v>
+        <v>0.008130141524979317</v>
       </c>
       <c r="G44">
-        <v>0.007117934652822733</v>
+        <v>0.0076760568404039</v>
       </c>
       <c r="H44">
-        <v>0.020140955026916263</v>
+        <v>0.02030330760719401</v>
       </c>
       <c r="I44">
-        <v>0.0020310862342879017</v>
+        <v>0.0015565214491938318</v>
       </c>
       <c r="J44">
-        <v>0.043374936050191125</v>
+        <v>0.043350253258958436</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -43353,7 +43532,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>corridor:44:butembo:kasese-uga</t>
+          <t>corridor:44:butembo:beni-cod</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -43363,33 +43542,33 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D45">
         <v>30</v>
       </c>
       <c r="E45">
-        <v>0.002966216009741285</v>
+        <v>0.002761100942238165</v>
       </c>
       <c r="F45">
-        <v>0.008071204783386715</v>
+        <v>0.008125095752590183</v>
       </c>
       <c r="G45">
-        <v>0.007384571167953435</v>
+        <v>0.006923387348404669</v>
       </c>
       <c r="H45">
-        <v>0.020017032108961774</v>
+        <v>0.020290785286753488</v>
       </c>
       <c r="I45">
-        <v>0.0019856633392102835</v>
+        <v>0.00206297360449538</v>
       </c>
       <c r="J45">
-        <v>0.03903230116776946</v>
+        <v>0.04222598903376526</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -43421,12 +43600,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>corridor:45:goma-cod:kampala-uga</t>
+          <t>corridor:45:bambu:kampala-uga</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -43438,26 +43617,26 @@
         <v>30</v>
       </c>
       <c r="E46">
-        <v>0.002999824043247834</v>
+        <v>0.002697580156124979</v>
       </c>
       <c r="F46">
-        <v>0.008070104040915183</v>
+        <v>0.008063051764023277</v>
       </c>
       <c r="G46">
-        <v>0.007468051852929203</v>
+        <v>0.006764436018809494</v>
       </c>
       <c r="H46">
-        <v>0.020014318893145783</v>
+        <v>0.020136791618205502</v>
       </c>
       <c r="I46">
-        <v>0.0018391957134823611</v>
+        <v>0.0017176606801707379</v>
       </c>
       <c r="J46">
-        <v>0.04222176098200819</v>
+        <v>0.03593932697202585</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -43489,43 +43668,43 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>corridor:46:miti-murhesa:kampala-uga</t>
+          <t>corridor:46:goma-cod:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>miti-murhesa</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D47">
         <v>30</v>
       </c>
       <c r="E47">
-        <v>0.00302696457253418</v>
+        <v>0.0029680417891685407</v>
       </c>
       <c r="F47">
-        <v>0.008061746356337274</v>
+        <v>0.008033249526172292</v>
       </c>
       <c r="G47">
-        <v>0.007535465665797686</v>
+        <v>0.007441119829860149</v>
       </c>
       <c r="H47">
-        <v>0.019993715064261175</v>
+        <v>0.020062799430107525</v>
       </c>
       <c r="I47">
-        <v>0.0019038903776436523</v>
+        <v>0.0018851508601080568</v>
       </c>
       <c r="J47">
-        <v>0.03809161905995875</v>
+        <v>0.041996978628116785</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -43557,43 +43736,43 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>corridor:47:miti-murhesa:kasese-uga</t>
+          <t>corridor:47:bambu:beni-cod</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>miti-murhesa</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D48">
         <v>30</v>
       </c>
       <c r="E48">
-        <v>0.002711272164641787</v>
+        <v>0.0029169808329018165</v>
       </c>
       <c r="F48">
-        <v>0.008003320140437448</v>
+        <v>0.007997964197460128</v>
       </c>
       <c r="G48">
-        <v>0.006751161363516417</v>
+        <v>0.007313388716630204</v>
       </c>
       <c r="H48">
-        <v>0.019849685301168624</v>
+        <v>0.019975227779149868</v>
       </c>
       <c r="I48">
-        <v>0.0016687253435851562</v>
+        <v>0.0023046023307807615</v>
       </c>
       <c r="J48">
-        <v>0.04165630204345164</v>
+        <v>0.04031690064358761</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -43625,7 +43804,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>corridor:48:kilo:bundibugyo-uga</t>
+          <t>corridor:48:kilo:kampala-uga</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -43635,33 +43814,33 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D49">
         <v>30</v>
       </c>
       <c r="E49">
-        <v>0.0028828781654738067</v>
+        <v>0.0030869625468540884</v>
       </c>
       <c r="F49">
-        <v>0.007999761114495657</v>
+        <v>0.007996867695904547</v>
       </c>
       <c r="G49">
-        <v>0.007177544340573161</v>
+        <v>0.007738556928652884</v>
       </c>
       <c r="H49">
-        <v>0.01984091087479531</v>
+        <v>0.01997250519785243</v>
       </c>
       <c r="I49">
-        <v>0.001746492912259029</v>
+        <v>0.0019306615451828934</v>
       </c>
       <c r="J49">
-        <v>0.04180829543410267</v>
+        <v>0.042052814805390165</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -43693,43 +43872,43 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>corridor:49:goma-cod:arua-uga</t>
+          <t>corridor:49:kilo:nebbi-uga</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>kilo</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D50">
         <v>30</v>
       </c>
       <c r="E50">
-        <v>0.0028290030722574744</v>
+        <v>0.002815721362600332</v>
       </c>
       <c r="F50">
-        <v>0.007993877766034052</v>
+        <v>0.007976076073243299</v>
       </c>
       <c r="G50">
-        <v>0.007043694470001555</v>
+        <v>0.0070600544320303105</v>
       </c>
       <c r="H50">
-        <v>0.01982640604270372</v>
+        <v>0.019920892154709158</v>
       </c>
       <c r="I50">
-        <v>0.0016184962560191808</v>
+        <v>0.001956233815972519</v>
       </c>
       <c r="J50">
-        <v>0.041811123101178745</v>
+        <v>0.04328982889117054</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -43761,43 +43940,43 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>corridor:50:nizi:beni-cod</t>
+          <t>corridor:50:goma-cod:nebbi-uga</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>nizi</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D51">
         <v>30</v>
       </c>
       <c r="E51">
-        <v>0.002964265235936736</v>
+        <v>0.0028080329489875433</v>
       </c>
       <c r="F51">
-        <v>0.007979683324545433</v>
+        <v>0.00795174060405468</v>
       </c>
       <c r="G51">
-        <v>0.007379725373273249</v>
+        <v>0.007040817734647403</v>
       </c>
       <c r="H51">
-        <v>0.01979141256348449</v>
+        <v>0.019860478352816707</v>
       </c>
       <c r="I51">
-        <v>0.001700272522619467</v>
+        <v>0.002303497064242352</v>
       </c>
       <c r="J51">
-        <v>0.03920759588832881</v>
+        <v>0.0471616963189368</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -43829,43 +44008,43 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>corridor:51:kilo:beni-cod</t>
+          <t>corridor:51:miti-murhesa:kampala-uga</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>kilo</t>
+          <t>miti-murhesa</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D52">
         <v>30</v>
       </c>
       <c r="E52">
-        <v>0.0027636218791129985</v>
+        <v>0.002980721344073456</v>
       </c>
       <c r="F52">
-        <v>0.007943736755445518</v>
+        <v>0.00793181040317939</v>
       </c>
       <c r="G52">
-        <v>0.006881244331427588</v>
+        <v>0.0074728367717477595</v>
       </c>
       <c r="H52">
-        <v>0.01970278797042238</v>
+        <v>0.019810999994700207</v>
       </c>
       <c r="I52">
-        <v>0.0014763767393302513</v>
+        <v>0.0016340821245132587</v>
       </c>
       <c r="J52">
-        <v>0.04005225312519262</v>
+        <v>0.042757776645511565</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -43897,43 +44076,43 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>corridor:52:kilo:kasese-uga</t>
+          <t>corridor:52:bambu:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>kilo</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D53">
         <v>30</v>
       </c>
       <c r="E53">
-        <v>0.002939240277028049</v>
+        <v>0.002668871809556994</v>
       </c>
       <c r="F53">
-        <v>0.007912160672771062</v>
+        <v>0.007918950601067454</v>
       </c>
       <c r="G53">
-        <v>0.007317560988202604</v>
+        <v>0.006692592465324332</v>
       </c>
       <c r="H53">
-        <v>0.019624933508132852</v>
+        <v>0.019779074000736363</v>
       </c>
       <c r="I53">
-        <v>0.0018917807676148398</v>
+        <v>0.0014712214192055375</v>
       </c>
       <c r="J53">
-        <v>0.038940141953057755</v>
+        <v>0.040525603585121125</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -43965,43 +44144,43 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>corridor:53:butembo:nebbi-uga</t>
+          <t>corridor:53:nizi:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>butembo</t>
+          <t>nizi</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D54">
         <v>30</v>
       </c>
       <c r="E54">
-        <v>0.002896284327627646</v>
+        <v>0.002970344773470357</v>
       </c>
       <c r="F54">
-        <v>0.007898422310050696</v>
+        <v>0.007916812374731491</v>
       </c>
       <c r="G54">
-        <v>0.007210849355384241</v>
+        <v>0.00744687994533258</v>
       </c>
       <c r="H54">
-        <v>0.019591060445456554</v>
+        <v>0.019773763992796817</v>
       </c>
       <c r="I54">
-        <v>0.002070995524055594</v>
+        <v>0.0018267951202627754</v>
       </c>
       <c r="J54">
-        <v>0.03944003878007347</v>
+        <v>0.0391235655311514</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -44033,43 +44212,43 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>corridor:54:goma-cod:nebbi-uga</t>
+          <t>corridor:54:bambu:kasese-uga</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D55">
         <v>30</v>
       </c>
       <c r="E55">
-        <v>0.00284876075269902</v>
+        <v>0.0031454086233342893</v>
       </c>
       <c r="F55">
-        <v>0.007893020209658985</v>
+        <v>0.00790638120557785</v>
       </c>
       <c r="G55">
-        <v>0.007092782818425181</v>
+        <v>0.007884733598589017</v>
       </c>
       <c r="H55">
-        <v>0.019577740869646337</v>
+        <v>0.019747868065662366</v>
       </c>
       <c r="I55">
-        <v>0.0020058959968129258</v>
+        <v>0.0021057835484370653</v>
       </c>
       <c r="J55">
-        <v>0.03794044182437606</v>
+        <v>0.03852983247889245</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -44101,43 +44280,43 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>corridor:55:bambu:beni-cod</t>
+          <t>corridor:55:kilo:arua-uga</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>kilo</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D56">
         <v>30</v>
       </c>
       <c r="E56">
-        <v>0.002919518350532113</v>
+        <v>0.00304220454384585</v>
       </c>
       <c r="F56">
-        <v>0.007885781628357735</v>
+        <v>0.007880648560680076</v>
       </c>
       <c r="G56">
-        <v>0.007268568604097025</v>
+        <v>0.0076266228561871485</v>
       </c>
       <c r="H56">
-        <v>0.0195598910020858</v>
+        <v>0.019683979639147753</v>
       </c>
       <c r="I56">
-        <v>0.0020982416358770435</v>
+        <v>0.0018498188421581965</v>
       </c>
       <c r="J56">
-        <v>0.04103833436051815</v>
+        <v>0.043875900176363315</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -44169,43 +44348,43 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>corridor:56:kilo:arua-uga</t>
+          <t>corridor:56:goma-cod:kasese-uga</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>kilo</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D57">
         <v>30</v>
       </c>
       <c r="E57">
-        <v>0.0026794581653525884</v>
+        <v>0.003169130129459574</v>
       </c>
       <c r="F57">
-        <v>0.007824052809558862</v>
+        <v>0.007864612484581951</v>
       </c>
       <c r="G57">
-        <v>0.0066721022582374445</v>
+        <v>0.007944054318325983</v>
       </c>
       <c r="H57">
-        <v>0.019407679063902866</v>
+        <v>0.019644164439568873</v>
       </c>
       <c r="I57">
-        <v>0.0018742235395998118</v>
+        <v>0.002417676492622753</v>
       </c>
       <c r="J57">
-        <v>0.03983832973283268</v>
+        <v>0.03686924375974461</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -44237,43 +44416,43 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>corridor:57:butembo:bundibugyo-uga</t>
+          <t>corridor:57:nizi:beni-cod</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>butembo</t>
+          <t>nizi</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D58">
         <v>30</v>
       </c>
       <c r="E58">
-        <v>0.0029658127649658528</v>
+        <v>0.002746685139402155</v>
       </c>
       <c r="F58">
-        <v>0.007809572414131216</v>
+        <v>0.007834762215712165</v>
       </c>
       <c r="G58">
-        <v>0.007383568737962282</v>
+        <v>0.006887313647931159</v>
       </c>
       <c r="H58">
-        <v>0.019371970574026537</v>
+        <v>0.019570047666818274</v>
       </c>
       <c r="I58">
-        <v>0.0018216334903385755</v>
+        <v>0.0019773417068834204</v>
       </c>
       <c r="J58">
-        <v>0.03964694132559633</v>
+        <v>0.03686928485677902</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -44305,43 +44484,43 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>corridor:58:nizi:arua-uga</t>
+          <t>corridor:58:miti-murhesa:nebbi-uga</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>nizi</t>
+          <t>miti-murhesa</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D59">
         <v>30</v>
       </c>
       <c r="E59">
-        <v>0.0028161227874957395</v>
+        <v>0.0028033145136891757</v>
       </c>
       <c r="F59">
-        <v>0.007799385470735554</v>
+        <v>0.007755839500948353</v>
       </c>
       <c r="G59">
-        <v>0.007011692758622234</v>
+        <v>0.007029011982497474</v>
       </c>
       <c r="H59">
-        <v>0.019346848345025758</v>
+        <v>0.019374068906622688</v>
       </c>
       <c r="I59">
-        <v>0.0021527480257039766</v>
+        <v>0.0016894071371955173</v>
       </c>
       <c r="J59">
-        <v>0.03738999809248955</v>
+        <v>0.04506619922585881</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -44373,7 +44552,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>corridor:59:butembo:beni-cod</t>
+          <t>corridor:59:butembo:arua-uga</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -44383,33 +44562,33 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D60">
         <v>30</v>
       </c>
       <c r="E60">
-        <v>0.002874053560650125</v>
+        <v>0.0027807819019262103</v>
       </c>
       <c r="F60">
-        <v>0.0077552415891767035</v>
+        <v>0.007730769920831854</v>
       </c>
       <c r="G60">
-        <v>0.007155620843306676</v>
+        <v>0.006972632877769225</v>
       </c>
       <c r="H60">
-        <v>0.019237984603597186</v>
+        <v>0.019311813845502956</v>
       </c>
       <c r="I60">
-        <v>0.0015960886164875705</v>
+        <v>0.001780853201348709</v>
       </c>
       <c r="J60">
-        <v>0.0397290483148042</v>
+        <v>0.03770510010166108</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -44441,12 +44620,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>corridor:60:goma-cod:bundibugyo-uga</t>
+          <t>corridor:60:kilo:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>kilo</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -44458,26 +44637,26 @@
         <v>30</v>
       </c>
       <c r="E61">
-        <v>0.0029333768169604313</v>
+        <v>0.003014014849821667</v>
       </c>
       <c r="F61">
-        <v>0.007738766942843367</v>
+        <v>0.007716679844077617</v>
       </c>
       <c r="G61">
-        <v>0.007302995550801578</v>
+        <v>0.007556114951172782</v>
       </c>
       <c r="H61">
-        <v>0.019197353961997482</v>
+        <v>0.019276823258474657</v>
       </c>
       <c r="I61">
-        <v>0.002113826548903264</v>
+        <v>0.001632307878839895</v>
       </c>
       <c r="J61">
-        <v>0.04367258678384024</v>
+        <v>0.03744864374175828</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -44509,43 +44688,43 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>corridor:61:bambu:bundibugyo-uga</t>
+          <t>corridor:61:miti-murhesa:beni-cod</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>miti-murhesa</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D62">
         <v>30</v>
       </c>
       <c r="E62">
-        <v>0.0029430467838043872</v>
+        <v>0.002519928132902971</v>
       </c>
       <c r="F62">
-        <v>0.007716591334032796</v>
+        <v>0.007698029728080397</v>
       </c>
       <c r="G62">
-        <v>0.007327016685413357</v>
+        <v>0.006319806901269265</v>
       </c>
       <c r="H62">
-        <v>0.019142661955798917</v>
+        <v>0.019230506044563306</v>
       </c>
       <c r="I62">
-        <v>0.0019755308676983633</v>
+        <v>0.0016384436173651762</v>
       </c>
       <c r="J62">
-        <v>0.039791083586982245</v>
+        <v>0.03885106071126117</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -44577,43 +44756,43 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>corridor:62:goma-cod:kasese-uga</t>
+          <t>corridor:62:bambu:nebbi-uga</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D63">
         <v>30</v>
       </c>
       <c r="E63">
-        <v>0.002796905767992547</v>
+        <v>0.0028232877052564442</v>
       </c>
       <c r="F63">
-        <v>0.00767757669112995</v>
+        <v>0.007649320956446215</v>
       </c>
       <c r="G63">
-        <v>0.006963945541292177</v>
+        <v>0.007078985649893704</v>
       </c>
       <c r="H63">
-        <v>0.019046434992530586</v>
+        <v>0.019109532549612368</v>
       </c>
       <c r="I63">
-        <v>0.0020588048892707404</v>
+        <v>0.0018363344309543978</v>
       </c>
       <c r="J63">
-        <v>0.049283570893681704</v>
+        <v>0.043637737653375794</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -44645,43 +44824,43 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>corridor:63:bambu:nebbi-uga</t>
+          <t>corridor:63:kilo:beni-cod</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>kilo</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D64">
         <v>30</v>
       </c>
       <c r="E64">
-        <v>0.002881574110656343</v>
+        <v>0.002826293275851488</v>
       </c>
       <c r="F64">
-        <v>0.0076527240222372395</v>
+        <v>0.007444085156304375</v>
       </c>
       <c r="G64">
-        <v>0.00717430459340368</v>
+        <v>0.007086505469572291</v>
       </c>
       <c r="H64">
-        <v>0.018985134000077397</v>
+        <v>0.01859970821153295</v>
       </c>
       <c r="I64">
-        <v>0.0019465263477377952</v>
+        <v>0.0017289297730197135</v>
       </c>
       <c r="J64">
-        <v>0.038295269411189395</v>
+        <v>0.04140206624718119</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -44713,43 +44892,43 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>corridor:64:miti-murhesa:arua-uga</t>
+          <t>corridor:64:kilo:kasese-uga</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>miti-murhesa</t>
+          <t>kilo</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D65">
         <v>30</v>
       </c>
       <c r="E65">
-        <v>0.0029594116020818517</v>
+        <v>0.0027471657296173346</v>
       </c>
       <c r="F65">
-        <v>0.007574358536086928</v>
+        <v>0.007411007252938445</v>
       </c>
       <c r="G65">
-        <v>0.007367668721658921</v>
+        <v>0.006888517718670689</v>
       </c>
       <c r="H65">
-        <v>0.018791827304817404</v>
+        <v>0.018517525239410138</v>
       </c>
       <c r="I65">
-        <v>0.0018921759864096277</v>
+        <v>0.001965558005404322</v>
       </c>
       <c r="J65">
-        <v>0.0362803906851146</v>
+        <v>0.038192040126588105</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -44781,43 +44960,43 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>corridor:65:butembo:kampala-uga</t>
+          <t>corridor:65:goma-cod:arua-uga</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>butembo</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D66">
         <v>30</v>
       </c>
       <c r="E66">
-        <v>0.0031623753037089974</v>
+        <v>0.0026959065523016745</v>
       </c>
       <c r="F66">
-        <v>0.00756670972052767</v>
+        <v>0.0073924555949739235</v>
       </c>
       <c r="G66">
-        <v>0.007871765533029873</v>
+        <v>0.006760247867125618</v>
       </c>
       <c r="H66">
-        <v>0.01877295839047441</v>
+        <v>0.01847143097717671</v>
       </c>
       <c r="I66">
-        <v>0.0022942651841674185</v>
+        <v>0.0020862923654499377</v>
       </c>
       <c r="J66">
-        <v>0.03629645524216742</v>
+        <v>0.03490935151153757</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -44849,43 +45028,43 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>corridor:66:kilo:nebbi-uga</t>
+          <t>corridor:66:butembo:kampala-uga</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>kilo</t>
+          <t>butembo</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D67">
         <v>30</v>
       </c>
       <c r="E67">
-        <v>0.0028544692621960133</v>
+        <v>0.0026528560781728105</v>
       </c>
       <c r="F67">
-        <v>0.0073600577545204215</v>
+        <v>0.007375241869799987</v>
       </c>
       <c r="G67">
-        <v>0.007106965376501684</v>
+        <v>0.0066525114617464465</v>
       </c>
       <c r="H67">
-        <v>0.018263086159490488</v>
+        <v>0.018428659273306808</v>
       </c>
       <c r="I67">
-        <v>0.0015953746275022913</v>
+        <v>0.002300845852606545</v>
       </c>
       <c r="J67">
-        <v>0.03555014814938943</v>
+        <v>0.04242449934097557</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.50× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 1 for this source zone; visibility-adjustment factor 2.51× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -45028,7 +45207,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-023</t>
+          <t>BDBV-CLAIM-024</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -45080,7 +45259,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-023</t>
+          <t>BDBV-CLAIM-024</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -45134,7 +45313,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-023</t>
+          <t>BDBV-CLAIM-024</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -45188,7 +45367,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-023</t>
+          <t>BDBV-CLAIM-024</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -45242,7 +45421,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-023</t>
+          <t>BDBV-CLAIM-024</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -45296,7 +45475,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-023</t>
+          <t>BDBV-CLAIM-024</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -45350,7 +45529,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-023</t>
+          <t>BDBV-CLAIM-024</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -45392,10 +45571,10 @@
       </c>
       <c r="D9"/>
       <c r="E9">
-        <v>0.4007872542276427</v>
+        <v>0.39797533849569694</v>
       </c>
       <c r="F9">
-        <v>0.4611775387681021</v>
+        <v>0.4577638723558707</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -45404,7 +45583,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-023</t>
+          <t>BDBV-CLAIM-024</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -45446,10 +45625,10 @@
       </c>
       <c r="D10"/>
       <c r="E10">
-        <v>2.6041684931341673</v>
+        <v>3.005236063491366</v>
       </c>
       <c r="F10">
-        <v>12.098434321451013</v>
+        <v>12.74823301250542</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -45458,7 +45637,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-023</t>
+          <t>BDBV-CLAIM-024</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -45500,10 +45679,10 @@
       </c>
       <c r="D11"/>
       <c r="E11">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="F11">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -45512,7 +45691,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-023</t>
+          <t>BDBV-CLAIM-024</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -45759,7 +45938,7 @@
         </is>
       </c>
       <c r="D16">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
       <c r="E16"/>
       <c r="F16"/>
@@ -45811,7 +45990,7 @@
         </is>
       </c>
       <c r="D17">
-        <v>0.035</v>
+        <v>0.033</v>
       </c>
       <c r="E17"/>
       <c r="F17"/>
@@ -45863,7 +46042,7 @@
         </is>
       </c>
       <c r="D18">
-        <v>0.958</v>
+        <v>0.959</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -47942,7 +48121,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-023</t>
+          <t>BDBV-CLAIM-024</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -47989,7 +48168,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-024</t>
+          <t>BDBV-CLAIM-025</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -47999,12 +48178,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>The May 23 public snapshot uses the CDC Current Situation page as the current official exact endpoint while retaining WHO 22 May and earlier values as dated conflict/cross-check evidence.</t>
+          <t>The May 23 public snapshot uses the CDC Current Situation page as the current official exact endpoint for confirmed cases, while the higher WHO 22 May suspected and suspected-deaths figures are the reconciled primaries under the higher-of-valid-primaries rule, and CDC's lower suspected/deaths plus earlier values are retained as dated conflict/cross-check evidence.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>confirmed total 88 (83 DRC + 5 Uganda), suspected DRC cases 746, suspected DRC deaths 176; CDC also reports nine confirmed DRC deaths and one confirmed Uganda death.</t>
+          <t>CDC reports confirmed total 88 (83 DRC + 5 Uganda), 746 suspected DRC cases, and 176 suspected DRC deaths, plus nine confirmed DRC deaths and one confirmed Uganda death. The reconciled endpoint takes CDC's 88 confirmed (the higher confirmed primary) and defers suspected and deaths to WHO 22 May (750 and 177, the higher valid primaries); CDC's 746 and 176 are retained as conflict anchors.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">

</xml_diff>

<commit_message>
Preserve May 25 source-review evidence without release trigger
</commit_message>
<xml_diff>
--- a/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
+++ b/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
@@ -125,7 +125,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -135,7 +135,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -1345,8 +1345,55 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BDBV-CLAIM-027</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Bdbv may25 source review boundary</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>May 25 source-review evidence can be archived for audit and partner context without creating a May 25 public snapshot route or promoting non-primary/watch claims into scored counts.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ECDC 25 May is accepted as regional cross-check only (snapshot_trigger=false); WHO AFRO hub is official context/readiness only (snapshot_trigger=false); IFRC requires browser/AIR capture when plain HTTP is challenged; Wikipedia remains watch-only unless confirmed by public-health authority.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>ECDC. Ebola virus disease outbreak in the Democratic Republic of the Congo and Uganda. Page last updated 25 May 2026 16:30.; WHO Regional Office for Africa. Ongoing outbreak in the Democratic Republic of the Congo / Bundibugyo virus disease outbreak hub. Updated 24 May 2026.; IFRC. Ebola: IFRC scales up response in eastern DRC as regional risks grow. 21 May 2026.; Wikipedia contributors. 2026 Ituri Province Ebola epidemic, live page observed by 25 May 2026 freshness check.; data/external_sources/freshness/bdbv-2026-2026-05-25.json generated by source_ingest.py --live-check --as-of 2026-05-25.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026; https://www.afro.who.int/health-topics/ebola-disease/outbreak-drc-26; https://www.ifrc.org/press-release/ebola-ifrc-scales-response-eastern-drc-regional-risks-grow; https://en.wikipedia.org/wiki/2026_Ituri_Province_Ebola_epidemic; restricted-local-review-not-redistributed</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Keep May 24 as the current publication-state route. Continue source review for DRC MoH table semantics, CDC traveler context, and future primary WHO/DRC/Uganda/CDC updates before any May 25 snapshot promotion.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Detailed audit IDs and review locators are withheld from this public export.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I24"/>
+  <autoFilter ref="A1:I25"/>
 </worksheet>
 </file>
 
@@ -3587,8 +3634,124 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>European Centre for Disease Prevention and Control</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>regional_body</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-05-25T16:30:00Z</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-05-25T18:36:38Z</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>public_bytes</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="J39"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>COD; UGA</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>who-afro-outbreak-hub-2026-05-24-live</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>World Health Organization, Regional Office for Africa</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>official_who_afro</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.afro.who.int/health-topics/ebola-disease/outbreak-drc-26</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-05-24T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-05-25T18:36:38Z</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>e7a8993d9d8526e69773fdc73f99b143e05b8d04184cdb69b02e2e34ab4cadb3</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>private_restricted_bytes</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>CC-BY-NC-SA-3.0-IGO</t>
+        </is>
+      </c>
+      <c r="J40"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>COD; UGA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L38"/>
+  <autoFilter ref="A1:L40"/>
 </worksheet>
 </file>
 
@@ -15699,8 +15862,270 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>source_data_report_date:ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>source_data_report_date</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="D116"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>regional_cross_check_only</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>regional_body</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>recorded</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Data/report date the source says the observation describes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>source_publication_date:ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>source_publication_date</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="D117"/>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>regional_cross_check_only</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>regional_body</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>recorded</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Date the source made the observation available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>source_retrieval_date:ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>source_retrieval_date</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>2026-05-25T18:36:38Z</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>regional_cross_check_only</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>regional_body</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>recorded</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Archive capture timestamp for this source edition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>source_data_report_date:who-afro-outbreak-hub-2026-05-24-live</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>source_data_report_date</t>
+        </is>
+      </c>
+      <c r="C119"/>
+      <c r="D119"/>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>who-afro-outbreak-hub-2026-05-24-live</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>context_only</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>official_who_afro</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>not_recorded</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Data/report date the source says the observation describes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>source_publication_date:who-afro-outbreak-hub-2026-05-24-live</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>source_publication_date</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="D120"/>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>who-afro-outbreak-hub-2026-05-24-live</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>context_only</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>official_who_afro</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>recorded</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Date the source made the observation available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>source_retrieval_date:who-afro-outbreak-hub-2026-05-24-live</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>source_retrieval_date</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>2026-05-25T18:36:38Z</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>who-afro-outbreak-hub-2026-05-24-live</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>context_only</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>official_who_afro</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>recorded</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Archive capture timestamp for this source edition.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I115"/>
+  <autoFilter ref="A1:I121"/>
 </worksheet>
 </file>
 
@@ -31715,34 +32140,34 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>snapshot:reported_counts:suspected</t>
+          <t>source:ecdc-bdbv-drc-uga-2026-05-25-live:cases_confirmed</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>snapshot_reconciled_metric</t>
+          <t>source_extracted_metric</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>suspected_cases</t>
-        </is>
-      </c>
-      <c r="D203"/>
+          <t>confirmed_cases</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>COD; UGA</t>
+        </is>
+      </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>2026-05-24T23:59:59Z</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="F203">
-        <v>904</v>
-      </c>
-      <c r="G203">
-        <v>395</v>
-      </c>
-      <c r="H203">
-        <v>904</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="G203"/>
+      <c r="H203"/>
       <c r="I203" t="inlineStr">
         <is>
           <t>count</t>
@@ -31750,37 +32175,33 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-24</t>
-        </is>
-      </c>
-      <c r="K203" t="inlineStr">
-        <is>
-          <t>afro-sitrep-01-2026-05-18-live; africa-cdc-phecs-2026-05-18-live; wikipedia-2026-ituri-epidemic-2026-05-20-live; ecdc-bdbv-drc-uga-2026-05-21-live; cdc-current-situation-2026-05-21; who-dg-remarks-bdbv-2026-05-22; drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24; cdc-current-situation-2026-05-24</t>
-        </is>
-      </c>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="K203"/>
       <c r="L203" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-026</t>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="M203" t="inlineStr">
         <is>
-          <t>reconciled_from_dated_sources</t>
+          <t>source_manifest_attested</t>
         </is>
       </c>
       <c r="N203" t="inlineStr">
         <is>
-          <t>snapshot_reconciled_range</t>
+          <t>source_extracted_metric</t>
         </is>
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
         </is>
       </c>
       <c r="P203" t="inlineStr">
         <is>
-          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
         </is>
       </c>
       <c r="Q203" t="inlineStr">
@@ -31790,7 +32211,7 @@
       </c>
       <c r="R203" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="S203"/>
@@ -31798,12 +32219,12 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>snapshot:reported_counts:confirmed</t>
+          <t>source:ecdc-bdbv-drc-uga-2026-05-25-live:cases_confirmed_drc</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>snapshot_reconciled_metric</t>
+          <t>source_extracted_metric</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -31811,21 +32232,21 @@
           <t>confirmed_cases</t>
         </is>
       </c>
-      <c r="D204"/>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>COD; UGA</t>
+        </is>
+      </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>2026-05-24T23:59:59Z</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="F204">
-        <v>106</v>
-      </c>
-      <c r="G204">
-        <v>10</v>
-      </c>
-      <c r="H204">
-        <v>106</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="G204"/>
+      <c r="H204"/>
       <c r="I204" t="inlineStr">
         <is>
           <t>count</t>
@@ -31833,37 +32254,33 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-24</t>
-        </is>
-      </c>
-      <c r="K204" t="inlineStr">
-        <is>
-          <t>who-pheic-2026-05-17-live; ecdc-bdbv-drc-uga-2026-05-19-live; wikipedia-2026-ituri-epidemic-2026-05-20-live; who-dg-remarks-bdbv-2026-05-20; cdc-current-situation-2026-05-21; who-dg-remarks-bdbv-2026-05-22; cdc-current-situation-2026-05-23; drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24; cdc-current-situation-2026-05-24</t>
-        </is>
-      </c>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="K204"/>
       <c r="L204" t="inlineStr">
         <is>
-          <t>BDBV-CLAIM-026</t>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>reconciled_from_dated_sources</t>
+          <t>source_manifest_attested</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
         <is>
-          <t>snapshot_reconciled_range</t>
+          <t>source_extracted_metric</t>
         </is>
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
         </is>
       </c>
       <c r="P204" t="inlineStr">
         <is>
-          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
         </is>
       </c>
       <c r="Q204" t="inlineStr">
@@ -31873,100 +32290,819 @@
       </c>
       <c r="R204" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
-        </is>
-      </c>
-      <c r="S204" t="inlineStr">
-        <is>
-          <t>WHO PHEIC deconfirmed the reported Kinshasa case; confirmed minimum excludes Kinshasa.</t>
-        </is>
-      </c>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="S204"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
+          <t>source:ecdc-bdbv-drc-uga-2026-05-25-live:cases_confirmed_uganda</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>confirmed_cases</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>COD; UGA</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="F205">
+        <v>7</v>
+      </c>
+      <c r="G205"/>
+      <c r="H205"/>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="K205"/>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>source_manifest_attested</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
+        </is>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
+        </is>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>public_bytes</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="S205"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>source:ecdc-bdbv-drc-uga-2026-05-25-live:cases_suspected</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>suspected_cases</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>COD; UGA</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="F206">
+        <v>904</v>
+      </c>
+      <c r="G206"/>
+      <c r="H206"/>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="K206"/>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>source_manifest_attested</t>
+        </is>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
+        </is>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
+        </is>
+      </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>public_bytes</t>
+        </is>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="S206"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>source:ecdc-bdbv-drc-uga-2026-05-25-live:contacts_followed_percent</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>contacts_followed_percent</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>COD; UGA</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="F207">
+        <v>20</v>
+      </c>
+      <c r="G207"/>
+      <c r="H207"/>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="K207"/>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>source_manifest_attested</t>
+        </is>
+      </c>
+      <c r="N207" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
+        </is>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
+        </is>
+      </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>public_bytes</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="S207"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>source:ecdc-bdbv-drc-uga-2026-05-25-live:contacts_identified_drc</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>contacts_identified_drc</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>COD; UGA</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="F208">
+        <v>1745</v>
+      </c>
+      <c r="G208"/>
+      <c r="H208"/>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="K208"/>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>source_manifest_attested</t>
+        </is>
+      </c>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
+        </is>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
+        </is>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>public_bytes</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="S208"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>source:ecdc-bdbv-drc-uga-2026-05-25-live:deaths_confirmed_drc</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>deaths</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>COD; UGA</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="F209">
+        <v>10</v>
+      </c>
+      <c r="G209"/>
+      <c r="H209"/>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="K209"/>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>source_manifest_attested</t>
+        </is>
+      </c>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
+        </is>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
+        </is>
+      </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>public_bytes</t>
+        </is>
+      </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="S209"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>source:ecdc-bdbv-drc-uga-2026-05-25-live:deaths_suspected</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>deaths</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>COD; UGA</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="F210">
+        <v>119</v>
+      </c>
+      <c r="G210"/>
+      <c r="H210"/>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="K210"/>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>source_manifest_attested</t>
+        </is>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
+        </is>
+      </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
+        </is>
+      </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>public_bytes</t>
+        </is>
+      </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="S210"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>source:ecdc-bdbv-drc-uga-2026-05-25-live:deaths_uganda</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>deaths</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>COD; UGA</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="F211">
+        <v>1</v>
+      </c>
+      <c r="G211"/>
+      <c r="H211"/>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="K211"/>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>source_manifest_attested</t>
+        </is>
+      </c>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>source_extracted_metric</t>
+        </is>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
+        </is>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
+        </is>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>public_bytes</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="S211"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>snapshot:reported_counts:suspected</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>snapshot_reconciled_metric</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>suspected_cases</t>
+        </is>
+      </c>
+      <c r="D212"/>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>2026-05-24T23:59:59Z</t>
+        </is>
+      </c>
+      <c r="F212">
+        <v>904</v>
+      </c>
+      <c r="G212">
+        <v>395</v>
+      </c>
+      <c r="H212">
+        <v>904</v>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>afro-sitrep-01-2026-05-18-live; africa-cdc-phecs-2026-05-18-live; wikipedia-2026-ituri-epidemic-2026-05-20-live; ecdc-bdbv-drc-uga-2026-05-21-live; cdc-current-situation-2026-05-21; who-dg-remarks-bdbv-2026-05-22; drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24; cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>BDBV-CLAIM-026</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>reconciled_from_dated_sources</t>
+        </is>
+      </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>snapshot_reconciled_range</t>
+        </is>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+        </is>
+      </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+        </is>
+      </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>public_bytes</t>
+        </is>
+      </c>
+      <c r="R212" t="inlineStr">
+        <is>
+          <t>public-domain-us-gov</t>
+        </is>
+      </c>
+      <c r="S212"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>snapshot:reported_counts:confirmed</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>snapshot_reconciled_metric</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>confirmed_cases</t>
+        </is>
+      </c>
+      <c r="D213"/>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>2026-05-24T23:59:59Z</t>
+        </is>
+      </c>
+      <c r="F213">
+        <v>106</v>
+      </c>
+      <c r="G213">
+        <v>10</v>
+      </c>
+      <c r="H213">
+        <v>106</v>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>who-pheic-2026-05-17-live; ecdc-bdbv-drc-uga-2026-05-19-live; wikipedia-2026-ituri-epidemic-2026-05-20-live; who-dg-remarks-bdbv-2026-05-20; cdc-current-situation-2026-05-21; who-dg-remarks-bdbv-2026-05-22; cdc-current-situation-2026-05-23; drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24; cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>BDBV-CLAIM-026</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>reconciled_from_dated_sources</t>
+        </is>
+      </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>snapshot_reconciled_range</t>
+        </is>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+        </is>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+        </is>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>public_bytes</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>public-domain-us-gov</t>
+        </is>
+      </c>
+      <c r="S213" t="inlineStr">
+        <is>
+          <t>WHO PHEIC deconfirmed the reported Kinshasa case; confirmed minimum excludes Kinshasa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
           <t>snapshot:reported_counts:deaths</t>
         </is>
       </c>
-      <c r="B205" t="inlineStr">
+      <c r="B214" t="inlineStr">
         <is>
           <t>snapshot_reconciled_metric</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr">
+      <c r="C214" t="inlineStr">
         <is>
           <t>deaths</t>
         </is>
       </c>
-      <c r="D205"/>
-      <c r="E205" t="inlineStr">
+      <c r="D214"/>
+      <c r="E214" t="inlineStr">
         <is>
           <t>2026-05-24T23:59:59Z</t>
         </is>
       </c>
-      <c r="F205">
+      <c r="F214">
         <v>179</v>
       </c>
-      <c r="G205">
+      <c r="G214">
         <v>106</v>
       </c>
-      <c r="H205">
+      <c r="H214">
         <v>179</v>
       </c>
-      <c r="I205" t="inlineStr">
+      <c r="I214" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="J205" t="inlineStr">
+      <c r="J214" t="inlineStr">
         <is>
           <t>drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24</t>
         </is>
       </c>
-      <c r="K205" t="inlineStr">
+      <c r="K214" t="inlineStr">
         <is>
           <t>afro-sitrep-01-2026-05-18-live; africa-cdc-phecs-2026-05-18-live; ecdc-bdbv-drc-uga-2026-05-21-live; wikipedia-2026-ituri-epidemic-2026-05-20-live; who-dg-remarks-bdbv-2026-05-20; cdc-current-situation-2026-05-21; who-dg-remarks-bdbv-2026-05-22; cdc-current-situation-2026-05-23; cdc-current-situation-2026-05-24; drc-moh-epidemie-dashboard-sitrep-009-graphql-2026-05-24</t>
         </is>
       </c>
-      <c r="L205" t="inlineStr">
+      <c r="L214" t="inlineStr">
         <is>
           <t>BDBV-CLAIM-026</t>
         </is>
       </c>
-      <c r="M205" t="inlineStr">
+      <c r="M214" t="inlineStr">
         <is>
           <t>reconciled_from_dated_sources</t>
         </is>
       </c>
-      <c r="N205" t="inlineStr">
+      <c r="N214" t="inlineStr">
         <is>
           <t>snapshot_reconciled_range</t>
         </is>
       </c>
-      <c r="O205" t="inlineStr">
+      <c r="O214" t="inlineStr">
         <is>
           <t>https://administration.sante.gouv.cd/graphql</t>
         </is>
       </c>
-      <c r="P205" t="inlineStr">
+      <c r="P214" t="inlineStr">
         <is>
           <t>f3d5149176d77cbf28d15c79bb7449b1a516c6b855ffe28d51b2adaef0f4bff5</t>
         </is>
       </c>
-      <c r="Q205" t="inlineStr">
+      <c r="Q214" t="inlineStr">
         <is>
           <t>private_restricted_bytes</t>
         </is>
       </c>
-      <c r="R205" t="inlineStr">
+      <c r="R214" t="inlineStr">
         <is>
           <t>publisher-terms-not-confirmed</t>
         </is>
       </c>
-      <c r="S205"/>
+      <c r="S214"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S205"/>
+  <autoFilter ref="A1:S214"/>
 </worksheet>
 </file>
 
@@ -41387,7 +42523,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-23:deaths_confirmed_drc</t>
+          <t>timeline:ecdc-bdbv-drc-uga-2026-05-25-live:cases_confirmed</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -41397,11 +42533,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>deaths</t>
+          <t>confirmed_cases</t>
         </is>
       </c>
       <c r="D185">
-        <v>9</v>
+        <v>101</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -41410,27 +42546,27 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-23</t>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-23</t>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="K185"/>
@@ -41438,7 +42574,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-23:deaths_suspected</t>
+          <t>timeline:ecdc-bdbv-drc-uga-2026-05-25-live:cases_confirmed_drc</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -41448,11 +42584,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>deaths</t>
+          <t>confirmed_cases</t>
         </is>
       </c>
       <c r="D186">
-        <v>176</v>
+        <v>101</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -41461,27 +42597,27 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-23</t>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-23</t>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="K186"/>
@@ -41489,7 +42625,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-23:deaths_suspected_drc</t>
+          <t>timeline:ecdc-bdbv-drc-uga-2026-05-25-live:cases_confirmed_uganda</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -41499,11 +42635,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>deaths</t>
+          <t>confirmed_cases</t>
         </is>
       </c>
       <c r="D187">
-        <v>176</v>
+        <v>7</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -41512,27 +42648,27 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-23</t>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-23</t>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="K187"/>
@@ -41540,7 +42676,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-23:deaths_uganda</t>
+          <t>timeline:ecdc-bdbv-drc-uga-2026-05-25-live:contacts_followed_percent</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -41550,11 +42686,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>deaths</t>
+          <t>contacts_followed_percent</t>
         </is>
       </c>
       <c r="D188">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -41563,27 +42699,27 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-23</t>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-23</t>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="K188"/>
@@ -41591,7 +42727,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-23:cases_suspected</t>
+          <t>timeline:ecdc-bdbv-drc-uga-2026-05-25-live:contacts_identified_drc</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -41601,11 +42737,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>suspected_cases</t>
+          <t>contacts_identified_drc</t>
         </is>
       </c>
       <c r="D189">
-        <v>746</v>
+        <v>1745</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -41614,27 +42750,27 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-23</t>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-23</t>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="K189"/>
@@ -41642,7 +42778,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-23:cases_suspected_drc</t>
+          <t>timeline:cdc-current-situation-2026-05-23:deaths_confirmed_drc</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -41652,11 +42788,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>suspected_cases</t>
+          <t>deaths</t>
         </is>
       </c>
       <c r="D190">
-        <v>746</v>
+        <v>9</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -41693,21 +42829,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-24:cases_confirmed</t>
+          <t>timeline:cdc-current-situation-2026-05-23:deaths_suspected</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>confirmed_cases</t>
+          <t>deaths</t>
         </is>
       </c>
       <c r="D191">
-        <v>106</v>
+        <v>176</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -41716,12 +42852,12 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-24</t>
+          <t>cdc-current-situation-2026-05-23</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+          <t>source_manifest:cdc-current-situation-2026-05-23</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -41731,7 +42867,7 @@
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
@@ -41744,21 +42880,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-24:cases_confirmed_drc</t>
+          <t>timeline:cdc-current-situation-2026-05-23:deaths_suspected_drc</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>confirmed_cases</t>
+          <t>deaths</t>
         </is>
       </c>
       <c r="D192">
-        <v>101</v>
+        <v>176</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -41767,12 +42903,12 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-24</t>
+          <t>cdc-current-situation-2026-05-23</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+          <t>source_manifest:cdc-current-situation-2026-05-23</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
@@ -41782,7 +42918,7 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -41795,21 +42931,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-24:cases_confirmed_total</t>
+          <t>timeline:cdc-current-situation-2026-05-23:deaths_uganda</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>confirmed_cases</t>
+          <t>deaths</t>
         </is>
       </c>
       <c r="D193">
-        <v>106</v>
+        <v>1</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -41818,12 +42954,12 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-24</t>
+          <t>cdc-current-situation-2026-05-23</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+          <t>source_manifest:cdc-current-situation-2026-05-23</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
@@ -41833,7 +42969,7 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -41846,21 +42982,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-24:cases_confirmed_uganda</t>
+          <t>timeline:ecdc-bdbv-drc-uga-2026-05-25-live:deaths_confirmed_drc</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>confirmed_cases</t>
+          <t>deaths</t>
         </is>
       </c>
       <c r="D194">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -41869,27 +43005,27 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-24</t>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="K194"/>
@@ -41897,21 +43033,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-24:cases_confirmed_united_states</t>
+          <t>timeline:ecdc-bdbv-drc-uga-2026-05-25-live:deaths_suspected</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>confirmed_cases</t>
+          <t>deaths</t>
         </is>
       </c>
       <c r="D195">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -41920,27 +43056,27 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-24</t>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="K195"/>
@@ -41948,21 +43084,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-24:new_confirmed_cases_uganda</t>
+          <t>timeline:ecdc-bdbv-drc-uga-2026-05-25-live:deaths_uganda</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>confirmed_cases</t>
+          <t>deaths</t>
         </is>
       </c>
       <c r="D196">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -41971,27 +43107,27 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-24</t>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="K196"/>
@@ -41999,21 +43135,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-24:deaths_confirmed_drc</t>
+          <t>timeline:cdc-current-situation-2026-05-23:cases_suspected</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>deaths</t>
+          <t>suspected_cases</t>
         </is>
       </c>
       <c r="D197">
-        <v>10</v>
+        <v>746</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -42022,12 +43158,12 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-24</t>
+          <t>cdc-current-situation-2026-05-23</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+          <t>source_manifest:cdc-current-situation-2026-05-23</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
@@ -42037,7 +43173,7 @@
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
@@ -42050,21 +43186,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-24:deaths_suspected</t>
+          <t>timeline:cdc-current-situation-2026-05-23:cases_suspected_drc</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>deaths</t>
+          <t>suspected_cases</t>
         </is>
       </c>
       <c r="D198">
-        <v>119</v>
+        <v>746</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -42073,12 +43209,12 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-24</t>
+          <t>cdc-current-situation-2026-05-23</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+          <t>source_manifest:cdc-current-situation-2026-05-23</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -42088,7 +43224,7 @@
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+          <t>1fa637ba0cb4ab11c50438b226bf00ebeca62757eda73a5738f4e6f231cdaed8</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
@@ -42101,21 +43237,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-24:deaths_suspected_drc</t>
+          <t>timeline:ecdc-bdbv-drc-uga-2026-05-25-live:cases_suspected</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>deaths</t>
+          <t>suspected_cases</t>
         </is>
       </c>
       <c r="D199">
-        <v>119</v>
+        <v>904</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -42124,27 +43260,27 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>cdc-current-situation-2026-05-24</t>
+          <t>ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+          <t>source_manifest:ecdc-bdbv-drc-uga-2026-05-25-live</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+          <t>https://www.ecdc.europa.eu/en/ebola-virus-disease-outbreak-democratic-republic-congo-and-uganda-19-may-2026</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+          <t>0636fc9b56903b84f738b1662879a6374d98946d3bb7fd58d20b4fed012ff57c</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>public-domain-us-gov</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="K199"/>
@@ -42152,7 +43288,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-24:deaths_uganda</t>
+          <t>timeline:cdc-current-situation-2026-05-24:cases_confirmed</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -42162,11 +43298,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>deaths</t>
+          <t>confirmed_cases</t>
         </is>
       </c>
       <c r="D200">
-        <v>1</v>
+        <v>106</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -42203,7 +43339,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>timeline:cdc-current-situation-2026-05-24:cases_suspected</t>
+          <t>timeline:cdc-current-situation-2026-05-24:cases_confirmed_drc</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -42213,11 +43349,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>suspected_cases</t>
+          <t>confirmed_cases</t>
         </is>
       </c>
       <c r="D201">
-        <v>904</v>
+        <v>101</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -42254,56 +43390,515 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
+          <t>timeline:cdc-current-situation-2026-05-24:cases_confirmed_total</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>confirmed_cases</t>
+        </is>
+      </c>
+      <c r="D202">
+        <v>106</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>public-domain-us-gov</t>
+        </is>
+      </c>
+      <c r="K202"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>timeline:cdc-current-situation-2026-05-24:cases_confirmed_uganda</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>confirmed_cases</t>
+        </is>
+      </c>
+      <c r="D203">
+        <v>5</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>public-domain-us-gov</t>
+        </is>
+      </c>
+      <c r="K203"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>timeline:cdc-current-situation-2026-05-24:cases_confirmed_united_states</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>confirmed_cases</t>
+        </is>
+      </c>
+      <c r="D204">
+        <v>0</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>public-domain-us-gov</t>
+        </is>
+      </c>
+      <c r="K204"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>timeline:cdc-current-situation-2026-05-24:new_confirmed_cases_uganda</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>confirmed_cases</t>
+        </is>
+      </c>
+      <c r="D205">
+        <v>3</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>public-domain-us-gov</t>
+        </is>
+      </c>
+      <c r="K205"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>timeline:cdc-current-situation-2026-05-24:deaths_confirmed_drc</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>deaths</t>
+        </is>
+      </c>
+      <c r="D206">
+        <v>10</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>public-domain-us-gov</t>
+        </is>
+      </c>
+      <c r="K206"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>timeline:cdc-current-situation-2026-05-24:deaths_suspected</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>deaths</t>
+        </is>
+      </c>
+      <c r="D207">
+        <v>119</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>public-domain-us-gov</t>
+        </is>
+      </c>
+      <c r="K207"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>timeline:cdc-current-situation-2026-05-24:deaths_suspected_drc</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>deaths</t>
+        </is>
+      </c>
+      <c r="D208">
+        <v>119</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>public-domain-us-gov</t>
+        </is>
+      </c>
+      <c r="K208"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>timeline:cdc-current-situation-2026-05-24:deaths_uganda</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>deaths</t>
+        </is>
+      </c>
+      <c r="D209">
+        <v>1</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>public-domain-us-gov</t>
+        </is>
+      </c>
+      <c r="K209"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>timeline:cdc-current-situation-2026-05-24:cases_suspected</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>suspected_cases</t>
+        </is>
+      </c>
+      <c r="D210">
+        <v>904</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>source_manifest:cdc-current-situation-2026-05-24</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>public-domain-us-gov</t>
+        </is>
+      </c>
+      <c r="K210"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
           <t>timeline:cdc-current-situation-2026-05-24:cases_suspected_drc</t>
         </is>
       </c>
-      <c r="B202" t="inlineStr">
+      <c r="B211" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
       </c>
-      <c r="C202" t="inlineStr">
+      <c r="C211" t="inlineStr">
         <is>
           <t>suspected_cases</t>
         </is>
       </c>
-      <c r="D202">
+      <c r="D211">
         <v>904</v>
       </c>
-      <c r="E202" t="inlineStr">
+      <c r="E211" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr">
+      <c r="F211" t="inlineStr">
         <is>
           <t>cdc-current-situation-2026-05-24</t>
         </is>
       </c>
-      <c r="G202" t="inlineStr">
+      <c r="G211" t="inlineStr">
         <is>
           <t>source_manifest:cdc-current-situation-2026-05-24</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr">
+      <c r="H211" t="inlineStr">
         <is>
           <t>https://www.cdc.gov/ebola/situation-summary/index.html</t>
         </is>
       </c>
-      <c r="I202" t="inlineStr">
+      <c r="I211" t="inlineStr">
         <is>
           <t>b33e81ab0e2af289ccde2ed4685a4a380f3397693ed2f6864e54a0f65227dc7d</t>
         </is>
       </c>
-      <c r="J202" t="inlineStr">
+      <c r="J211" t="inlineStr">
         <is>
           <t>public-domain-us-gov</t>
         </is>
       </c>
-      <c r="K202"/>
+      <c r="K211"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K202"/>
+  <autoFilter ref="A1:K211"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fix ECDC-25 conflict-anchor id to canonical form (corridor cascade)
The 25 May ECDC conflict anchor was listed with the manifest -live suffix
(ecdc-bdbv-drc-uga-2026-05-25-live) in the reconciliation conflict trails and
NUMBERS_AUDIT, while repo convention (every other trail entry) uses the
canonical suffix-stripped id. The LOVS gates tolerated it (they canonicalize),
but the figure did not resolve into the visibility cascade, so the corridor
range was computed without ECDC-25 in the uncertainty set. With the canonical
id it resolves: corridor 50% range is now 0.6-21.2% lower / 1.8-48.2% upper
(was 0.6-21.1 / 1.9-49.1). Updated contract, README, NUMBERS_AUDIT,
evidence-chains, and the contract test. Surfaced by the website sync's source
resolver.
</commit_message>
<xml_diff>
--- a/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
+++ b/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
@@ -1081,7 +1081,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>headline confirmed total 112; officially zone-attributed corridor source-load total 79 across 11 DRC MoH source zones; 33 confirmed cases remain unallocated headline context; current 66-corridor adjusted 50% range is 0.6-21.1% lower bounds and 1.9-49.1% upper bounds.</t>
+          <t>headline confirmed total 112; officially zone-attributed corridor source-load total 79 across 11 DRC MoH source zones; 33 confirmed cases remain unallocated headline context; current 66-corridor adjusted 50% range is 0.6-21.2% lower bounds and 1.8-48.2% upper bounds.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -47020,7 +47020,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>corridor:01:rwampara:beni-cod</t>
+          <t>corridor:01:rwampara:nebbi-uga</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -47030,29 +47030,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D2">
         <v>30</v>
       </c>
       <c r="E2">
-        <v>0.08705872476656829</v>
+        <v>0.0861708114385285</v>
       </c>
       <c r="F2">
-        <v>0.23849877729636965</v>
+        <v>0.23315469335620254</v>
       </c>
       <c r="G2">
-        <v>0.20200901575875693</v>
+        <v>0.20028631694823662</v>
       </c>
       <c r="H2">
-        <v>0.490855636804455</v>
+        <v>0.48234065943233195</v>
       </c>
       <c r="I2">
-        <v>0.05827234299127523</v>
+        <v>0.06427581319980569</v>
       </c>
       <c r="J2">
-        <v>0.7360585970208364</v>
+        <v>0.7474537035483133</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -47088,7 +47088,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>corridor:02:rwampara:kampala-uga</t>
+          <t>corridor:02:rwampara:kasese-uga</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -47098,29 +47098,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D3">
         <v>30</v>
       </c>
       <c r="E3">
-        <v>0.09106071850782033</v>
+        <v>0.08768171124595683</v>
       </c>
       <c r="F3">
-        <v>0.23180304927763629</v>
+        <v>0.2275794037963691</v>
       </c>
       <c r="G3">
-        <v>0.21064783365598588</v>
+        <v>0.2035618016305265</v>
       </c>
       <c r="H3">
-        <v>0.47969244396961136</v>
+        <v>0.47295633103988544</v>
       </c>
       <c r="I3">
-        <v>0.05967373659336905</v>
+        <v>0.04459460740614488</v>
       </c>
       <c r="J3">
-        <v>0.7123311692401879</v>
+        <v>0.7478981260349676</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -47156,7 +47156,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>corridor:03:rwampara:nebbi-uga</t>
+          <t>corridor:03:rwampara:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -47166,29 +47166,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D4">
         <v>30</v>
       </c>
       <c r="E4">
-        <v>0.08277521513409741</v>
+        <v>0.08233054224498484</v>
       </c>
       <c r="F4">
-        <v>0.22641515556489766</v>
+        <v>0.22543492066869397</v>
       </c>
       <c r="G4">
-        <v>0.19270105652080258</v>
+        <v>0.19192499609422323</v>
       </c>
       <c r="H4">
-        <v>0.47060445029291187</v>
+        <v>0.46931800011005115</v>
       </c>
       <c r="I4">
-        <v>0.058851102281542125</v>
+        <v>0.06964130796312437</v>
       </c>
       <c r="J4">
-        <v>0.7381007215516742</v>
+        <v>0.6990237917928565</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -47224,7 +47224,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>corridor:04:rwampara:kasese-uga</t>
+          <t>corridor:04:rwampara:beni-cod</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -47234,29 +47234,29 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D5">
         <v>30</v>
       </c>
       <c r="E5">
-        <v>0.0777667177980044</v>
+        <v>0.08664306873590838</v>
       </c>
       <c r="F5">
-        <v>0.22125498504359012</v>
+        <v>0.222887038238157</v>
       </c>
       <c r="G5">
-        <v>0.18173566771392538</v>
+        <v>0.20131080198240825</v>
       </c>
       <c r="H5">
-        <v>0.46181259202543024</v>
+        <v>0.4649794327839667</v>
       </c>
       <c r="I5">
-        <v>0.04687532836669559</v>
+        <v>0.05425688863966508</v>
       </c>
       <c r="J5">
-        <v>0.7431942191372538</v>
+        <v>0.7101842045533336</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -47292,7 +47292,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>corridor:05:rwampara:bundibugyo-uga</t>
+          <t>corridor:05:rwampara:arua-uga</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -47302,29 +47302,29 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D6">
         <v>30</v>
       </c>
       <c r="E6">
-        <v>0.08994167609221052</v>
+        <v>0.09176382815314144</v>
       </c>
       <c r="F6">
-        <v>0.21814102710172356</v>
+        <v>0.2196720235905948</v>
       </c>
       <c r="G6">
-        <v>0.2082377356100764</v>
+        <v>0.2123714082943657</v>
       </c>
       <c r="H6">
-        <v>0.4564648825278334</v>
+        <v>0.45947010738720273</v>
       </c>
       <c r="I6">
-        <v>0.06843498725883312</v>
+        <v>0.0602209036243418</v>
       </c>
       <c r="J6">
-        <v>0.7351838704184875</v>
+        <v>0.7146926481656625</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -47360,7 +47360,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>corridor:06:rwampara:arua-uga</t>
+          <t>corridor:06:rwampara:kampala-uga</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -47370,29 +47370,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D7">
         <v>30</v>
       </c>
       <c r="E7">
-        <v>0.08738592639250203</v>
+        <v>0.08396936085735776</v>
       </c>
       <c r="F7">
-        <v>0.21691539014958308</v>
+        <v>0.2119043283318027</v>
       </c>
       <c r="G7">
-        <v>0.20271776834032668</v>
+        <v>0.19549948212877702</v>
       </c>
       <c r="H7">
-        <v>0.4543515172508829</v>
+        <v>0.44602874389977687</v>
       </c>
       <c r="I7">
-        <v>0.0606006699211846</v>
+        <v>0.056360235565877555</v>
       </c>
       <c r="J7">
-        <v>0.7294259710737864</v>
+        <v>0.7142786607680277</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -47428,43 +47428,43 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>corridor:07:bunia:kampala-uga</t>
+          <t>corridor:07:mongbwalu:nebbi-uga</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>bunia</t>
+          <t>mongbwalu</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D8">
         <v>30</v>
       </c>
       <c r="E8">
-        <v>0.04246356113673297</v>
+        <v>0.03855467933328152</v>
       </c>
       <c r="F8">
-        <v>0.11942130278737001</v>
+        <v>0.11620932868289471</v>
       </c>
       <c r="G8">
-        <v>0.10192493852909751</v>
+        <v>0.09291440432184914</v>
       </c>
       <c r="H8">
-        <v>0.270266609097878</v>
+        <v>0.2639086114886541</v>
       </c>
       <c r="I8">
-        <v>0.028409667809219823</v>
+        <v>0.025175207094245807</v>
       </c>
       <c r="J8">
-        <v>0.46391565999619183</v>
+        <v>0.46361890390099453</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.48× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.48× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -47496,7 +47496,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>corridor:08:bunia:bundibugyo-uga</t>
+          <t>corridor:08:bunia:kampala-uga</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -47506,29 +47506,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D9">
         <v>30</v>
       </c>
       <c r="E9">
-        <v>0.04372720174962935</v>
+        <v>0.04147908524423352</v>
       </c>
       <c r="F9">
-        <v>0.11776659374999701</v>
+        <v>0.11562806950949953</v>
       </c>
       <c r="G9">
-        <v>0.10485843323233299</v>
+        <v>0.09974219409345544</v>
       </c>
       <c r="H9">
-        <v>0.2668648630838556</v>
+        <v>0.2627072705721946</v>
       </c>
       <c r="I9">
-        <v>0.024824081936019447</v>
+        <v>0.025907663365721464</v>
       </c>
       <c r="J9">
-        <v>0.47074791691760753</v>
+        <v>0.4462554570998926</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -47564,7 +47564,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>corridor:09:bunia:beni-cod</t>
+          <t>corridor:09:bunia:arua-uga</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -47574,29 +47574,29 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D10">
         <v>30</v>
       </c>
       <c r="E10">
-        <v>0.043721416421617726</v>
+        <v>0.04179480816556652</v>
       </c>
       <c r="F10">
-        <v>0.11772211441413447</v>
+        <v>0.11558245421258095</v>
       </c>
       <c r="G10">
-        <v>0.1048450145946053</v>
+        <v>0.10047743392001213</v>
       </c>
       <c r="H10">
-        <v>0.2667733722448983</v>
+        <v>0.26261295488077974</v>
       </c>
       <c r="I10">
-        <v>0.03158643596552796</v>
+        <v>0.027913949480659363</v>
       </c>
       <c r="J10">
-        <v>0.4736878533835456</v>
+        <v>0.4647552683750245</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -47649,22 +47649,22 @@
         <v>30</v>
       </c>
       <c r="E11">
-        <v>0.0444155412592947</v>
+        <v>0.04186956091160368</v>
       </c>
       <c r="F11">
-        <v>0.11571118127048804</v>
+        <v>0.11539491748492897</v>
       </c>
       <c r="G11">
-        <v>0.10645391938867926</v>
+        <v>0.10065158442248001</v>
       </c>
       <c r="H11">
-        <v>0.2626253665816084</v>
+        <v>0.26222507759010427</v>
       </c>
       <c r="I11">
-        <v>0.03078606866593397</v>
+        <v>0.021242880051839726</v>
       </c>
       <c r="J11">
-        <v>0.4883461510873249</v>
+        <v>0.46678607844486947</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -47700,12 +47700,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>corridor:11:bunia:kasese-uga</t>
+          <t>corridor:11:mongbwalu:kasese-uga</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>bunia</t>
+          <t>mongbwalu</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -47717,26 +47717,26 @@
         <v>30</v>
       </c>
       <c r="E12">
-        <v>0.04410979236313228</v>
+        <v>0.04042920346327944</v>
       </c>
       <c r="F12">
-        <v>0.11505461271845879</v>
+        <v>0.11242435593909272</v>
       </c>
       <c r="G12">
-        <v>0.10574531651674063</v>
+        <v>0.09729451222456448</v>
       </c>
       <c r="H12">
-        <v>0.26126870223516685</v>
+        <v>0.2560645676658191</v>
       </c>
       <c r="I12">
-        <v>0.028827859136638982</v>
+        <v>0.027413735537554062</v>
       </c>
       <c r="J12">
-        <v>0.4349056791496498</v>
+        <v>0.43705126759089724</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.48× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.48× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -47768,7 +47768,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>corridor:12:bunia:arua-uga</t>
+          <t>corridor:12:bunia:kasese-uga</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -47778,29 +47778,29 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D13">
         <v>30</v>
       </c>
       <c r="E13">
-        <v>0.04061609325636212</v>
+        <v>0.04024586283096926</v>
       </c>
       <c r="F13">
-        <v>0.11396739072964437</v>
+        <v>0.11159467152136757</v>
       </c>
       <c r="G13">
-        <v>0.09762606642203506</v>
+        <v>0.09686667859605977</v>
       </c>
       <c r="H13">
-        <v>0.25901826950891554</v>
+        <v>0.25433876336268857</v>
       </c>
       <c r="I13">
-        <v>0.02387539752522782</v>
+        <v>0.03067229187569909</v>
       </c>
       <c r="J13">
-        <v>0.4461622227370582</v>
+        <v>0.4576157180833162</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -47836,7 +47836,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>corridor:13:mongbwalu:beni-cod</t>
+          <t>corridor:13:mongbwalu:kampala-uga</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -47846,29 +47846,29 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D14">
         <v>30</v>
       </c>
       <c r="E14">
-        <v>0.03710996846095013</v>
+        <v>0.04066526892293623</v>
       </c>
       <c r="F14">
-        <v>0.10964681236938656</v>
+        <v>0.11152320362817797</v>
       </c>
       <c r="G14">
-        <v>0.08943382811819442</v>
+        <v>0.09784524147753831</v>
       </c>
       <c r="H14">
-        <v>0.250034224844084</v>
+        <v>0.254190125108517</v>
       </c>
       <c r="I14">
-        <v>0.03385391457147437</v>
+        <v>0.026605224754838577</v>
       </c>
       <c r="J14">
-        <v>0.46993004228955715</v>
+        <v>0.46394166684739413</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -47904,43 +47904,43 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>corridor:14:mongbwalu:nebbi-uga</t>
+          <t>corridor:14:bunia:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>mongbwalu</t>
+          <t>bunia</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D15">
         <v>30</v>
       </c>
       <c r="E15">
-        <v>0.042080228665137914</v>
+        <v>0.043769887053943884</v>
       </c>
       <c r="F15">
-        <v>0.10683766833988695</v>
+        <v>0.11103027985574987</v>
       </c>
       <c r="G15">
-        <v>0.10103406480576219</v>
+        <v>0.10506919313252691</v>
       </c>
       <c r="H15">
-        <v>0.24415829376737277</v>
+        <v>0.2531634176228099</v>
       </c>
       <c r="I15">
-        <v>0.027024110522923</v>
+        <v>0.024326153776741695</v>
       </c>
       <c r="J15">
-        <v>0.4126434945709156</v>
+        <v>0.44860424323610526</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.48× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.48× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -47972,7 +47972,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>corridor:15:mongbwalu:bundibugyo-uga</t>
+          <t>corridor:15:mongbwalu:beni-cod</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -47982,29 +47982,29 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D16">
         <v>30</v>
       </c>
       <c r="E16">
-        <v>0.04202426525540365</v>
+        <v>0.03750471405393857</v>
       </c>
       <c r="F16">
-        <v>0.10608468442723934</v>
+        <v>0.10749948779872281</v>
       </c>
       <c r="G16">
-        <v>0.10090394584352139</v>
+        <v>0.09045541125798737</v>
       </c>
       <c r="H16">
-        <v>0.24257853052369338</v>
+        <v>0.24578444055142545</v>
       </c>
       <c r="I16">
-        <v>0.025730387416915464</v>
+        <v>0.027237694409312466</v>
       </c>
       <c r="J16">
-        <v>0.4196281916748507</v>
+        <v>0.4271444488438072</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -48040,43 +48040,43 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>corridor:16:mongbwalu:arua-uga</t>
+          <t>corridor:16:bunia:beni-cod</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>mongbwalu</t>
+          <t>bunia</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D17">
         <v>30</v>
       </c>
       <c r="E17">
-        <v>0.03933542211197083</v>
+        <v>0.04228950663900796</v>
       </c>
       <c r="F17">
-        <v>0.10546729596630738</v>
+        <v>0.10704031678368539</v>
       </c>
       <c r="G17">
-        <v>0.09463884639695044</v>
+        <v>0.10162893993380431</v>
       </c>
       <c r="H17">
-        <v>0.24128195279119546</v>
+        <v>0.24482175888282368</v>
       </c>
       <c r="I17">
-        <v>0.024899713049719586</v>
+        <v>0.026598690800271954</v>
       </c>
       <c r="J17">
-        <v>0.45412776873008587</v>
+        <v>0.4232379895804849</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>zone-attributed confirmed count 14 for this source zone; visibility-adjustment factor 2.48× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
+          <t>zone-attributed confirmed count 15 for this source zone; visibility-adjustment factor 2.48× reflects under-reporting in source zone; raw risk likely understates true hazard</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -48108,7 +48108,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>corridor:17:mongbwalu:kasese-uga</t>
+          <t>corridor:17:mongbwalu:arua-uga</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -48118,29 +48118,29 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D18">
         <v>30</v>
       </c>
       <c r="E18">
-        <v>0.03674677955972819</v>
+        <v>0.03798452079077774</v>
       </c>
       <c r="F18">
-        <v>0.10253826350865747</v>
+        <v>0.1055578744412985</v>
       </c>
       <c r="G18">
-        <v>0.08858269196104879</v>
+        <v>0.09157962059775004</v>
       </c>
       <c r="H18">
-        <v>0.2351121722828113</v>
+        <v>0.24170839592150667</v>
       </c>
       <c r="I18">
-        <v>0.02446060018301769</v>
+        <v>0.0239669463086208</v>
       </c>
       <c r="J18">
-        <v>0.43434320993589176</v>
+        <v>0.4664322846035496</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -48176,7 +48176,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>corridor:18:mongbwalu:kampala-uga</t>
+          <t>corridor:18:mongbwalu:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -48186,29 +48186,29 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D19">
         <v>30</v>
       </c>
       <c r="E19">
-        <v>0.03673769680232783</v>
+        <v>0.03778298943272401</v>
       </c>
       <c r="F19">
-        <v>0.10176519464035952</v>
+        <v>0.10384450964700326</v>
       </c>
       <c r="G19">
-        <v>0.08856139661635878</v>
+        <v>0.09110754488962608</v>
       </c>
       <c r="H19">
-        <v>0.23347872961217356</v>
+        <v>0.23810062900458037</v>
       </c>
       <c r="I19">
-        <v>0.019766568129704724</v>
+        <v>0.027747327225511372</v>
       </c>
       <c r="J19">
-        <v>0.45173277256401556</v>
+        <v>0.39188625277934763</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -48244,7 +48244,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>corridor:19:nyankunde:nebbi-uga</t>
+          <t>corridor:19:nyankunde:kasese-uga</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -48254,29 +48254,29 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D20">
         <v>30</v>
       </c>
       <c r="E20">
-        <v>0.02943619547001522</v>
+        <v>0.031304381068294335</v>
       </c>
       <c r="F20">
-        <v>0.08644089973446445</v>
+        <v>0.08779786212598711</v>
       </c>
       <c r="G20">
-        <v>0.07134929740790441</v>
+        <v>0.07585358277896675</v>
       </c>
       <c r="H20">
-        <v>0.20067080506318333</v>
+        <v>0.2038133127969261</v>
       </c>
       <c r="I20">
-        <v>0.017249897635217455</v>
+        <v>0.017690770792813504</v>
       </c>
       <c r="J20">
-        <v>0.37720643415082816</v>
+        <v>0.3619871650097016</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -48312,7 +48312,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>corridor:20:nyankunde:kampala-uga</t>
+          <t>corridor:20:nyankunde:beni-cod</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -48322,29 +48322,29 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D21">
         <v>30</v>
       </c>
       <c r="E21">
-        <v>0.03143620060038951</v>
+        <v>0.03171837340940942</v>
       </c>
       <c r="F21">
-        <v>0.08597135121230412</v>
+        <v>0.08476753807336304</v>
       </c>
       <c r="G21">
-        <v>0.0760830743974528</v>
+        <v>0.07683287603147732</v>
       </c>
       <c r="H21">
-        <v>0.19965252253419963</v>
+        <v>0.19723709872212672</v>
       </c>
       <c r="I21">
-        <v>0.026413643415756798</v>
+        <v>0.0227792144919888</v>
       </c>
       <c r="J21">
-        <v>0.3875565167376865</v>
+        <v>0.3495642294984912</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -48380,7 +48380,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>corridor:21:nyankunde:bundibugyo-uga</t>
+          <t>corridor:21:nyankunde:kampala-uga</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -48390,29 +48390,29 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D22">
         <v>30</v>
       </c>
       <c r="E22">
-        <v>0.033545219747423194</v>
+        <v>0.030540418665822744</v>
       </c>
       <c r="F22">
-        <v>0.08571847788474835</v>
+        <v>0.08438962198493272</v>
       </c>
       <c r="G22">
-        <v>0.08105927552190084</v>
+        <v>0.07404478785217791</v>
       </c>
       <c r="H22">
-        <v>0.19910390583267018</v>
+        <v>0.19641470100450442</v>
       </c>
       <c r="I22">
-        <v>0.02488466056117501</v>
+        <v>0.019203507671592176</v>
       </c>
       <c r="J22">
-        <v>0.3750758008783629</v>
+        <v>0.3838230566411262</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -48448,7 +48448,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>corridor:22:nyankunde:arua-uga</t>
+          <t>corridor:22:nyankunde:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -48458,29 +48458,29 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D23">
         <v>30</v>
       </c>
       <c r="E23">
-        <v>0.03209426849587091</v>
+        <v>0.030399316276041116</v>
       </c>
       <c r="F23">
-        <v>0.08294965297286142</v>
+        <v>0.08407821789447709</v>
       </c>
       <c r="G23">
-        <v>0.07763750605795702</v>
+        <v>0.07371053738981273</v>
       </c>
       <c r="H23">
-        <v>0.19308102183167064</v>
+        <v>0.19573661412777732</v>
       </c>
       <c r="I23">
-        <v>0.01788217072461529</v>
+        <v>0.021457583298788</v>
       </c>
       <c r="J23">
-        <v>0.34301640031334013</v>
+        <v>0.358453978352833</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -48516,7 +48516,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>corridor:23:nyankunde:beni-cod</t>
+          <t>corridor:23:nyankunde:nebbi-uga</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -48526,29 +48526,29 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D24">
         <v>30</v>
       </c>
       <c r="E24">
-        <v>0.02866534159045145</v>
+        <v>0.030329334773183142</v>
       </c>
       <c r="F24">
-        <v>0.08246390394965086</v>
+        <v>0.08357711531060097</v>
       </c>
       <c r="G24">
-        <v>0.0695208928496309</v>
+        <v>0.07354468946695608</v>
       </c>
       <c r="H24">
-        <v>0.19202205699078656</v>
+        <v>0.19464486287655744</v>
       </c>
       <c r="I24">
-        <v>0.016730935405880526</v>
+        <v>0.014570952055622657</v>
       </c>
       <c r="J24">
-        <v>0.364088590258062</v>
+        <v>0.32281669746439295</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -48584,7 +48584,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>corridor:24:nyankunde:kasese-uga</t>
+          <t>corridor:24:nyankunde:arua-uga</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -48594,29 +48594,29 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D25">
         <v>30</v>
       </c>
       <c r="E25">
-        <v>0.03081565613688028</v>
+        <v>0.028578262502321705</v>
       </c>
       <c r="F25">
-        <v>0.08049341862637019</v>
+        <v>0.0757669915923353</v>
       </c>
       <c r="G25">
-        <v>0.07461586978106036</v>
+        <v>0.06938957908843438</v>
       </c>
       <c r="H25">
-        <v>0.18771637107786493</v>
+        <v>0.17751379634539563</v>
       </c>
       <c r="I25">
-        <v>0.026248954426468973</v>
+        <v>0.021112935786516</v>
       </c>
       <c r="J25">
-        <v>0.3381175600724034</v>
+        <v>0.3190059046148159</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -48652,7 +48652,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>corridor:25:katwa:nebbi-uga</t>
+          <t>corridor:25:katwa:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -48662,29 +48662,29 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D26">
         <v>30</v>
       </c>
       <c r="E26">
-        <v>0.006029262723708073</v>
+        <v>0.006127400208913586</v>
       </c>
       <c r="F26">
-        <v>0.017114033671260853</v>
+        <v>0.0168408512437718</v>
       </c>
       <c r="G26">
-        <v>0.014870934354623777</v>
+        <v>0.015128788346279537</v>
       </c>
       <c r="H26">
-        <v>0.04186515305349886</v>
+        <v>0.04125072266262608</v>
       </c>
       <c r="I26">
-        <v>0.004470615331371439</v>
+        <v>0.004388490481047946</v>
       </c>
       <c r="J26">
-        <v>0.0770842786162016</v>
+        <v>0.08183093712788367</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -48720,7 +48720,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>corridor:26:katwa:arua-uga</t>
+          <t>corridor:26:katwa:kasese-uga</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -48730,29 +48730,29 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D27">
         <v>30</v>
       </c>
       <c r="E27">
-        <v>0.005522357235792252</v>
+        <v>0.00556423388622837</v>
       </c>
       <c r="F27">
-        <v>0.016224882815260827</v>
+        <v>0.01656759676464939</v>
       </c>
       <c r="G27">
-        <v>0.013625786217095454</v>
+        <v>0.013744050643107991</v>
       </c>
       <c r="H27">
-        <v>0.039716335710117456</v>
+        <v>0.04058965567523373</v>
       </c>
       <c r="I27">
-        <v>0.0035817052958976416</v>
+        <v>0.003889156206565628</v>
       </c>
       <c r="J27">
-        <v>0.07992818660808958</v>
+        <v>0.08557353521823044</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -48788,7 +48788,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>corridor:27:katwa:bundibugyo-uga</t>
+          <t>corridor:27:katwa:kampala-uga</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -48798,29 +48798,29 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D28">
         <v>30</v>
       </c>
       <c r="E28">
-        <v>0.005763485989899592</v>
+        <v>0.00571138519466724</v>
       </c>
       <c r="F28">
-        <v>0.015897712364671857</v>
+        <v>0.016458424878468436</v>
       </c>
       <c r="G28">
-        <v>0.01421820486301828</v>
+        <v>0.014105980367321913</v>
       </c>
       <c r="H28">
-        <v>0.038924937410599686</v>
+        <v>0.04032548046029999</v>
       </c>
       <c r="I28">
-        <v>0.00412817012599338</v>
+        <v>0.0032961116192571803</v>
       </c>
       <c r="J28">
-        <v>0.07530722471772157</v>
+        <v>0.08227064654779426</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -48856,7 +48856,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>corridor:28:katwa:kasese-uga</t>
+          <t>corridor:28:katwa:beni-cod</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -48866,29 +48866,29 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D29">
         <v>30</v>
       </c>
       <c r="E29">
-        <v>0.00569825474665156</v>
+        <v>0.005665299126924983</v>
       </c>
       <c r="F29">
-        <v>0.015708110329420072</v>
+        <v>0.016137547052658407</v>
       </c>
       <c r="G29">
-        <v>0.014057962115334166</v>
+        <v>0.01399263950136656</v>
       </c>
       <c r="H29">
-        <v>0.03846612710006386</v>
+        <v>0.039548733878884995</v>
       </c>
       <c r="I29">
-        <v>0.0030738801757677933</v>
+        <v>0.0033705192295240497</v>
       </c>
       <c r="J29">
-        <v>0.08554865711076257</v>
+        <v>0.0787241376496719</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -48924,7 +48924,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>corridor:29:katwa:beni-cod</t>
+          <t>corridor:29:katwa:arua-uga</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -48934,29 +48934,29 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D30">
         <v>30</v>
       </c>
       <c r="E30">
-        <v>0.006051188152445097</v>
+        <v>0.005760920437457601</v>
       </c>
       <c r="F30">
-        <v>0.01568874267670098</v>
+        <v>0.01564371888735397</v>
       </c>
       <c r="G30">
-        <v>0.014924768457324877</v>
+        <v>0.014227802835785092</v>
       </c>
       <c r="H30">
-        <v>0.03841925323098799</v>
+        <v>0.03835261291771347</v>
       </c>
       <c r="I30">
-        <v>0.003838228121916951</v>
+        <v>0.004405736887256273</v>
       </c>
       <c r="J30">
-        <v>0.08215270653449197</v>
+        <v>0.07717071840257644</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -48992,7 +48992,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>corridor:30:katwa:kampala-uga</t>
+          <t>corridor:30:katwa:nebbi-uga</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -49002,29 +49002,29 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D31">
         <v>30</v>
       </c>
       <c r="E31">
-        <v>0.005782262522765952</v>
+        <v>0.005519371147358398</v>
       </c>
       <c r="F31">
-        <v>0.015216280256187209</v>
+        <v>0.01552589721826908</v>
       </c>
       <c r="G31">
-        <v>0.014264327261309523</v>
+        <v>0.013633690221780848</v>
       </c>
       <c r="H31">
-        <v>0.03727535911897989</v>
+        <v>0.03806709980880993</v>
       </c>
       <c r="I31">
-        <v>0.0033384218962603934</v>
+        <v>0.003119740043250069</v>
       </c>
       <c r="J31">
-        <v>0.07811576042493965</v>
+        <v>0.07892668631060598</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -49060,39 +49060,39 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>corridor:31:bambu:beni-cod</t>
+          <t>corridor:31:goma-cod:kasese-uga</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D32">
         <v>30</v>
       </c>
       <c r="E32">
-        <v>0.0031221041967082197</v>
+        <v>0.002911020622911431</v>
       </c>
       <c r="F32">
-        <v>0.008698068132782094</v>
+        <v>0.008708366339810258</v>
       </c>
       <c r="G32">
-        <v>0.007717131898621776</v>
+        <v>0.007204585754623377</v>
       </c>
       <c r="H32">
-        <v>0.021411044648201427</v>
+        <v>0.021460131514392883</v>
       </c>
       <c r="I32">
-        <v>0.0017828154968101114</v>
+        <v>0.002213739571223128</v>
       </c>
       <c r="J32">
-        <v>0.0431818978878234</v>
+        <v>0.04056094344785632</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -49128,39 +49128,39 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>corridor:32:miti-murhesa:beni-cod</t>
+          <t>corridor:32:butembo:nebbi-uga</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>miti-murhesa</t>
+          <t>butembo</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D33">
         <v>30</v>
       </c>
       <c r="E33">
-        <v>0.003256550077390147</v>
+        <v>0.0027769798502101373</v>
       </c>
       <c r="F33">
-        <v>0.008690654774771961</v>
+        <v>0.008633599440103473</v>
       </c>
       <c r="G33">
-        <v>0.008048651456418393</v>
+        <v>0.006873526257886398</v>
       </c>
       <c r="H33">
-        <v>0.02139291864359122</v>
+        <v>0.021277062424142124</v>
       </c>
       <c r="I33">
-        <v>0.002208850691779005</v>
+        <v>0.0016525413787399719</v>
       </c>
       <c r="J33">
-        <v>0.0397230321776111</v>
+        <v>0.03899275669757771</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -49196,39 +49196,39 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>corridor:33:goma-cod:arua-uga</t>
+          <t>corridor:33:miti-murhesa:kasese-uga</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>miti-murhesa</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D34">
         <v>30</v>
       </c>
       <c r="E34">
-        <v>0.0029781199558879257</v>
+        <v>0.0029900129594525315</v>
       </c>
       <c r="F34">
-        <v>0.008646396347219365</v>
+        <v>0.00847697711451803</v>
       </c>
       <c r="G34">
-        <v>0.00736201964546096</v>
+        <v>0.007399652921270428</v>
       </c>
       <c r="H34">
-        <v>0.021284669747048707</v>
+        <v>0.020893505827646625</v>
       </c>
       <c r="I34">
-        <v>0.001720505229708283</v>
+        <v>0.0017305897295624153</v>
       </c>
       <c r="J34">
-        <v>0.038678795905731755</v>
+        <v>0.04136198023793251</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
@@ -49264,39 +49264,39 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>corridor:34:goma-cod:kampala-uga</t>
+          <t>corridor:34:butembo:arua-uga</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>butembo</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D35">
         <v>30</v>
       </c>
       <c r="E35">
-        <v>0.003111181616698544</v>
+        <v>0.003004206625567968</v>
       </c>
       <c r="F35">
-        <v>0.008628383148852753</v>
+        <v>0.008424640775256842</v>
       </c>
       <c r="G35">
-        <v>0.007690196297224505</v>
+        <v>0.007434701480319217</v>
       </c>
       <c r="H35">
-        <v>0.021240605916741817</v>
+        <v>0.02076531908923876</v>
       </c>
       <c r="I35">
-        <v>0.0016110230461111126</v>
+        <v>0.0014445621581179958</v>
       </c>
       <c r="J35">
-        <v>0.043150308180892</v>
+        <v>0.03973256156228256</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
@@ -49332,12 +49332,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>corridor:35:bambu:bundibugyo-uga</t>
+          <t>corridor:35:nizi:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>nizi</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -49349,22 +49349,22 @@
         <v>30</v>
       </c>
       <c r="E36">
-        <v>0.0030884074123188887</v>
+        <v>0.003111941625778658</v>
       </c>
       <c r="F36">
-        <v>0.008588026182462571</v>
+        <v>0.008402719753006271</v>
       </c>
       <c r="G36">
-        <v>0.007634031778964906</v>
+        <v>0.0077007053534820236</v>
       </c>
       <c r="H36">
-        <v>0.02114189671152855</v>
+        <v>0.020711624541566498</v>
       </c>
       <c r="I36">
-        <v>0.0020051565560971376</v>
+        <v>0.0017674417542844795</v>
       </c>
       <c r="J36">
-        <v>0.03964300574013423</v>
+        <v>0.038221794937289805</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -49400,7 +49400,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>corridor:36:butembo:bundibugyo-uga</t>
+          <t>corridor:36:butembo:kampala-uga</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -49410,29 +49410,29 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D37">
         <v>30</v>
       </c>
       <c r="E37">
-        <v>0.003025775628822114</v>
+        <v>0.002898657102272467</v>
       </c>
       <c r="F37">
-        <v>0.008571115858547917</v>
+        <v>0.00831048662323794</v>
       </c>
       <c r="G37">
-        <v>0.007479562809800805</v>
+        <v>0.0071740522491085534</v>
       </c>
       <c r="H37">
-        <v>0.021100531187123267</v>
+        <v>0.020485685215592936</v>
       </c>
       <c r="I37">
-        <v>0.0021199327441538463</v>
+        <v>0.0024156585156788397</v>
       </c>
       <c r="J37">
-        <v>0.04196071647036671</v>
+        <v>0.03953263154110449</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -49468,39 +49468,39 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>corridor:37:nizi:bundibugyo-uga</t>
+          <t>corridor:37:goma-cod:arua-uga</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>nizi</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D38">
         <v>30</v>
       </c>
       <c r="E38">
-        <v>0.002797267917861973</v>
+        <v>0.0027125515817747747</v>
       </c>
       <c r="F38">
-        <v>0.00846270517529632</v>
+        <v>0.008284511161890662</v>
       </c>
       <c r="G38">
-        <v>0.006915872271437584</v>
+        <v>0.006714374614320118</v>
       </c>
       <c r="H38">
-        <v>0.020835318333113584</v>
+        <v>0.020422048400997733</v>
       </c>
       <c r="I38">
-        <v>0.0018633454289880586</v>
+        <v>0.0015261556624343033</v>
       </c>
       <c r="J38">
-        <v>0.04328965085234269</v>
+        <v>0.04121550107288618</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -49536,12 +49536,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>corridor:38:bambu:nebbi-uga</t>
+          <t>corridor:38:nizi:nebbi-uga</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>nizi</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -49553,22 +49553,22 @@
         <v>30</v>
       </c>
       <c r="E39">
-        <v>0.0027165842894116</v>
+        <v>0.002681493416460179</v>
       </c>
       <c r="F39">
-        <v>0.008462033120420043</v>
+        <v>0.008183525990654555</v>
       </c>
       <c r="G39">
-        <v>0.006716793549505717</v>
+        <v>0.0066376497183083805</v>
       </c>
       <c r="H39">
-        <v>0.020833674557079906</v>
+        <v>0.020174624300513644</v>
       </c>
       <c r="I39">
-        <v>0.0020833936544929683</v>
+        <v>0.0014926750968995012</v>
       </c>
       <c r="J39">
-        <v>0.03946198024192364</v>
+        <v>0.039228799255843605</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -49604,39 +49604,39 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>corridor:39:kilo:kampala-uga</t>
+          <t>corridor:39:nizi:beni-cod</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>kilo</t>
+          <t>nizi</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D40">
         <v>30</v>
       </c>
       <c r="E40">
-        <v>0.002827091182153685</v>
+        <v>0.0028326663994584778</v>
       </c>
       <c r="F40">
-        <v>0.00844775188405536</v>
+        <v>0.00815823939873217</v>
       </c>
       <c r="G40">
-        <v>0.00698945216246713</v>
+        <v>0.00701107122667835</v>
       </c>
       <c r="H40">
-        <v>0.020798732145144022</v>
+        <v>0.020112663896618338</v>
       </c>
       <c r="I40">
-        <v>0.002402073067513322</v>
+        <v>0.0015343125999103453</v>
       </c>
       <c r="J40">
-        <v>0.04203889492505474</v>
+        <v>0.04046059631457021</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -49672,12 +49672,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>corridor:40:goma-cod:kasese-uga</t>
+          <t>corridor:40:butembo:kasese-uga</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>butembo</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -49689,22 +49689,22 @@
         <v>30</v>
       </c>
       <c r="E41">
-        <v>0.003098245083166251</v>
+        <v>0.002747567807505402</v>
       </c>
       <c r="F41">
-        <v>0.008421295606099832</v>
+        <v>0.008154445449094133</v>
       </c>
       <c r="G41">
-        <v>0.007658292806589306</v>
+        <v>0.006800874406568735</v>
       </c>
       <c r="H41">
-        <v>0.02073400424273225</v>
+        <v>0.020103367023304758</v>
       </c>
       <c r="I41">
-        <v>0.0019012551291241716</v>
+        <v>0.0016545850906405566</v>
       </c>
       <c r="J41">
-        <v>0.043972182665138686</v>
+        <v>0.04190231971566359</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -49740,39 +49740,39 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>corridor:41:nizi:kasese-uga</t>
+          <t>corridor:41:bambu:arua-uga</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>nizi</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D42">
         <v>30</v>
       </c>
       <c r="E42">
-        <v>0.0028569543753373394</v>
+        <v>0.0029994938796520376</v>
       </c>
       <c r="F42">
-        <v>0.008399426913836133</v>
+        <v>0.008147226747461322</v>
       </c>
       <c r="G42">
-        <v>0.007063127009692638</v>
+        <v>0.007423064501010185</v>
       </c>
       <c r="H42">
-        <v>0.02068049618046927</v>
+        <v>0.020085678474308588</v>
       </c>
       <c r="I42">
-        <v>0.001940933593041583</v>
+        <v>0.0019885435545158206</v>
       </c>
       <c r="J42">
-        <v>0.043335795648454876</v>
+        <v>0.03889536735459872</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -49808,39 +49808,39 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>corridor:42:kilo:beni-cod</t>
+          <t>corridor:42:miti-murhesa:nebbi-uga</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>kilo</t>
+          <t>miti-murhesa</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D43">
         <v>30</v>
       </c>
       <c r="E43">
-        <v>0.003208969909536785</v>
+        <v>0.003061304197971737</v>
       </c>
       <c r="F43">
-        <v>0.008396225534473778</v>
+        <v>0.00814381727681368</v>
       </c>
       <c r="G43">
-        <v>0.007931333169932525</v>
+        <v>0.00757568403154249</v>
       </c>
       <c r="H43">
-        <v>0.020672662243381656</v>
+        <v>0.020077321716829383</v>
       </c>
       <c r="I43">
-        <v>0.002451028146972545</v>
+        <v>0.0016647585017794454</v>
       </c>
       <c r="J43">
-        <v>0.03828745231097391</v>
+        <v>0.03886426325038798</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -49876,39 +49876,39 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>corridor:43:miti-murhesa:kasese-uga</t>
+          <t>corridor:43:goma-cod:nebbi-uga</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>miti-murhesa</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D44">
         <v>30</v>
       </c>
       <c r="E44">
-        <v>0.0029666436131503826</v>
+        <v>0.0031340416283216765</v>
       </c>
       <c r="F44">
-        <v>0.008357295677379833</v>
+        <v>0.008075152624742232</v>
       </c>
       <c r="G44">
-        <v>0.007333712327801806</v>
+        <v>0.00775526629452003</v>
       </c>
       <c r="H44">
-        <v>0.020577406853998614</v>
+        <v>0.01990905693022571</v>
       </c>
       <c r="I44">
-        <v>0.0017909766821187448</v>
+        <v>0.002243955437822981</v>
       </c>
       <c r="J44">
-        <v>0.04221199332021168</v>
+        <v>0.03925743592923069</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -49944,7 +49944,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>corridor:44:kilo:nebbi-uga</t>
+          <t>corridor:44:kilo:kasese-uga</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -49954,29 +49954,29 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D45">
         <v>30</v>
       </c>
       <c r="E45">
-        <v>0.002842466144925393</v>
+        <v>0.0027076980614253177</v>
       </c>
       <c r="F45">
-        <v>0.008306902670088073</v>
+        <v>0.008070258181662043</v>
       </c>
       <c r="G45">
-        <v>0.007027383918706276</v>
+        <v>0.006702384988596155</v>
       </c>
       <c r="H45">
-        <v>0.02045409216417554</v>
+        <v>0.019897061858827808</v>
       </c>
       <c r="I45">
-        <v>0.001971915409122316</v>
+        <v>0.0018949255081115225</v>
       </c>
       <c r="J45">
-        <v>0.040177434293513725</v>
+        <v>0.03846409821761752</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
@@ -50012,39 +50012,39 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>corridor:45:nizi:arua-uga</t>
+          <t>corridor:45:bambu:nebbi-uga</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>nizi</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>nebbi-uga</t>
         </is>
       </c>
       <c r="D46">
         <v>30</v>
       </c>
       <c r="E46">
-        <v>0.0029776446786048127</v>
+        <v>0.0029941551171358827</v>
       </c>
       <c r="F46">
-        <v>0.00827436066103368</v>
+        <v>0.008062710206497403</v>
       </c>
       <c r="G46">
-        <v>0.007360847692718359</v>
+        <v>0.007409881598903129</v>
       </c>
       <c r="H46">
-        <v>0.020374455899091842</v>
+        <v>0.019878564189878323</v>
       </c>
       <c r="I46">
-        <v>0.0020194029902177533</v>
+        <v>0.0023605934928140225</v>
       </c>
       <c r="J46">
-        <v>0.0390744440809115</v>
+        <v>0.03849962672911588</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -50080,39 +50080,39 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>corridor:46:butembo:kampala-uga</t>
+          <t>corridor:46:goma-cod:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>butembo</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D47">
         <v>30</v>
       </c>
       <c r="E47">
-        <v>0.0027549525104297867</v>
+        <v>0.002966610048958429</v>
       </c>
       <c r="F47">
-        <v>0.008222628255700165</v>
+        <v>0.008058011311337127</v>
       </c>
       <c r="G47">
-        <v>0.006811466224796531</v>
+        <v>0.007341863257414205</v>
       </c>
       <c r="H47">
-        <v>0.020247848860154932</v>
+        <v>0.01986704842779069</v>
       </c>
       <c r="I47">
-        <v>0.002002134515076684</v>
+        <v>0.00193425911064469</v>
       </c>
       <c r="J47">
-        <v>0.042430507815804784</v>
+        <v>0.03944581553096073</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
@@ -50148,39 +50148,39 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>corridor:47:goma-cod:bundibugyo-uga</t>
+          <t>corridor:47:miti-murhesa:beni-cod</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>miti-murhesa</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D48">
         <v>30</v>
       </c>
       <c r="E48">
-        <v>0.002882502947612553</v>
+        <v>0.002837150359859514</v>
       </c>
       <c r="F48">
-        <v>0.008194900129801702</v>
+        <v>0.008035393220128945</v>
       </c>
       <c r="G48">
-        <v>0.0071261552896609015</v>
+        <v>0.007022145861493551</v>
       </c>
       <c r="H48">
-        <v>0.02017998389325623</v>
+        <v>0.019811615320896397</v>
       </c>
       <c r="I48">
-        <v>0.0014343817285406735</v>
+        <v>0.0016272804773103918</v>
       </c>
       <c r="J48">
-        <v>0.03991556549220518</v>
+        <v>0.0417257099987222</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
@@ -50216,39 +50216,39 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>corridor:48:butembo:kasese-uga</t>
+          <t>corridor:48:bambu:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>butembo</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D49">
         <v>30</v>
       </c>
       <c r="E49">
-        <v>0.002899735778643775</v>
+        <v>0.0027221893165624844</v>
       </c>
       <c r="F49">
-        <v>0.008156775375274178</v>
+        <v>0.008025112676473323</v>
       </c>
       <c r="G49">
-        <v>0.007168667109143045</v>
+        <v>0.006738183364620509</v>
       </c>
       <c r="H49">
-        <v>0.020086668634671817</v>
+        <v>0.019786420160049306</v>
       </c>
       <c r="I49">
-        <v>0.001765702714835879</v>
+        <v>0.0018923716266919608</v>
       </c>
       <c r="J49">
-        <v>0.039438828983039326</v>
+        <v>0.04067091464985655</v>
       </c>
       <c r="K49" t="inlineStr">
         <is>
@@ -50284,12 +50284,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>corridor:49:goma-cod:beni-cod</t>
+          <t>corridor:49:butembo:beni-cod</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>butembo</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -50301,22 +50301,22 @@
         <v>30</v>
       </c>
       <c r="E50">
-        <v>0.0027436075367688606</v>
+        <v>0.0029779299971779694</v>
       </c>
       <c r="F50">
-        <v>0.00813573057807132</v>
+        <v>0.007993848855793961</v>
       </c>
       <c r="G50">
-        <v>0.006783473348184826</v>
+        <v>0.007369816645196731</v>
       </c>
       <c r="H50">
-        <v>0.02003515768678027</v>
+        <v>0.019709793462212938</v>
       </c>
       <c r="I50">
-        <v>0.0019484543771382619</v>
+        <v>0.00181708380560561</v>
       </c>
       <c r="J50">
-        <v>0.04366249567204285</v>
+        <v>0.03931941479325931</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
@@ -50352,12 +50352,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>corridor:50:butembo:arua-uga</t>
+          <t>corridor:50:nizi:arua-uga</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>butembo</t>
+          <t>nizi</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -50369,22 +50369,22 @@
         <v>30</v>
       </c>
       <c r="E51">
-        <v>0.00289673081900102</v>
+        <v>0.002573515092590184</v>
       </c>
       <c r="F51">
-        <v>0.008093538488025936</v>
+        <v>0.007966550348283807</v>
       </c>
       <c r="G51">
-        <v>0.0071612541418274445</v>
+        <v>0.006370874666990878</v>
       </c>
       <c r="H51">
-        <v>0.019931878246767426</v>
+        <v>0.01964288498845579</v>
       </c>
       <c r="I51">
-        <v>0.0016809985549575749</v>
+        <v>0.0019758723489192026</v>
       </c>
       <c r="J51">
-        <v>0.04244857346914838</v>
+        <v>0.042497226842963434</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -50420,39 +50420,39 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>corridor:51:miti-murhesa:kampala-uga</t>
+          <t>corridor:51:bambu:kasese-uga</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>miti-murhesa</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D52">
         <v>30</v>
       </c>
       <c r="E52">
-        <v>0.0029401286142527183</v>
+        <v>0.00270874962073242</v>
       </c>
       <c r="F52">
-        <v>0.008060259325341046</v>
+        <v>0.007945705918331214</v>
       </c>
       <c r="G52">
-        <v>0.0072683082461652004</v>
+        <v>0.006704981285868744</v>
       </c>
       <c r="H52">
-        <v>0.019850402601428535</v>
+        <v>0.019591793108546057</v>
       </c>
       <c r="I52">
-        <v>0.001797781260891848</v>
+        <v>0.0017099558870529636</v>
       </c>
       <c r="J52">
-        <v>0.03851102703520781</v>
+        <v>0.040311579752921115</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -50488,39 +50488,39 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>corridor:52:bambu:arua-uga</t>
+          <t>corridor:52:goma-cod:kampala-uga</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D53">
         <v>30</v>
       </c>
       <c r="E53">
-        <v>0.002865544957359273</v>
+        <v>0.002937977495464733</v>
       </c>
       <c r="F53">
-        <v>0.008007505347331828</v>
+        <v>0.00791077263458917</v>
       </c>
       <c r="G53">
-        <v>0.0070843200252671545</v>
+        <v>0.007271156988672728</v>
       </c>
       <c r="H53">
-        <v>0.019721262395209938</v>
+        <v>0.019506162869570853</v>
       </c>
       <c r="I53">
-        <v>0.0015405355995758848</v>
+        <v>0.0015259490592032937</v>
       </c>
       <c r="J53">
-        <v>0.03672115158663102</v>
+        <v>0.04355956758414158</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -50556,12 +50556,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>corridor:53:miti-murhesa:nebbi-uga</t>
+          <t>corridor:53:kilo:nebbi-uga</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>miti-murhesa</t>
+          <t>kilo</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -50573,22 +50573,22 @@
         <v>30</v>
       </c>
       <c r="E54">
-        <v>0.0029536944459469527</v>
+        <v>0.0025676185126164985</v>
       </c>
       <c r="F54">
-        <v>0.007960826510511443</v>
+        <v>0.007868621059145403</v>
       </c>
       <c r="G54">
-        <v>0.007301771191140616</v>
+        <v>0.0063563051772850265</v>
       </c>
       <c r="H54">
-        <v>0.01960697825032018</v>
+        <v>0.01940283456752373</v>
       </c>
       <c r="I54">
-        <v>0.0016862635592489572</v>
+        <v>0.0016564750458324922</v>
       </c>
       <c r="J54">
-        <v>0.045197930386536175</v>
+        <v>0.03677402473147005</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -50624,39 +50624,39 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>corridor:54:bambu:kampala-uga</t>
+          <t>corridor:54:miti-murhesa:arua-uga</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>miti-murhesa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D55">
         <v>30</v>
       </c>
       <c r="E55">
-        <v>0.0028077086856141686</v>
+        <v>0.0027868684736187532</v>
       </c>
       <c r="F55">
-        <v>0.007901485678099562</v>
+        <v>0.007841801348761585</v>
       </c>
       <c r="G55">
-        <v>0.006941632095260497</v>
+        <v>0.00689795184472039</v>
       </c>
       <c r="H55">
-        <v>0.01946168095865239</v>
+        <v>0.019337083521810405</v>
       </c>
       <c r="I55">
-        <v>0.0021553033511651945</v>
+        <v>0.0017127846529912062</v>
       </c>
       <c r="J55">
-        <v>0.04097440772519585</v>
+        <v>0.03838966632456429</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
@@ -50692,39 +50692,39 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>corridor:55:butembo:beni-cod</t>
+          <t>corridor:55:bambu:kampala-uga</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>butembo</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>beni-cod</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D56">
         <v>30</v>
       </c>
       <c r="E56">
-        <v>0.0029325884804620728</v>
+        <v>0.002695763743499391</v>
       </c>
       <c r="F56">
-        <v>0.0078658503326898</v>
+        <v>0.007827990157414616</v>
       </c>
       <c r="G56">
-        <v>0.007249708704873986</v>
+        <v>0.006672903334783625</v>
       </c>
       <c r="H56">
-        <v>0.01937442245861365</v>
+        <v>0.0193032265603717</v>
       </c>
       <c r="I56">
-        <v>0.0023275583555744496</v>
+        <v>0.0021490354133257674</v>
       </c>
       <c r="J56">
-        <v>0.04310662676624314</v>
+        <v>0.04054210634480244</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
@@ -50760,7 +50760,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>corridor:56:kilo:kasese-uga</t>
+          <t>corridor:56:kilo:beni-cod</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -50770,29 +50770,29 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D57">
         <v>30</v>
       </c>
       <c r="E57">
-        <v>0.002964790671466655</v>
+        <v>0.003089733434463643</v>
       </c>
       <c r="F57">
-        <v>0.007845522849790815</v>
+        <v>0.007797896708572921</v>
       </c>
       <c r="G57">
-        <v>0.007329141803465333</v>
+        <v>0.007645875573836641</v>
       </c>
       <c r="H57">
-        <v>0.019324644695648402</v>
+        <v>0.019229449244770908</v>
       </c>
       <c r="I57">
-        <v>0.001979182980043831</v>
+        <v>0.0016800255774773844</v>
       </c>
       <c r="J57">
-        <v>0.03709606445309815</v>
+        <v>0.034479825340189424</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
@@ -50828,39 +50828,39 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>corridor:57:miti-murhesa:arua-uga</t>
+          <t>corridor:57:kilo:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>miti-murhesa</t>
+          <t>kilo</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D58">
         <v>30</v>
       </c>
       <c r="E58">
-        <v>0.002787974005366123</v>
+        <v>0.002629641493342244</v>
       </c>
       <c r="F58">
-        <v>0.007811983261174604</v>
+        <v>0.0077950978062735765</v>
       </c>
       <c r="G58">
-        <v>0.006892941705632205</v>
+        <v>0.006509547825961637</v>
       </c>
       <c r="H58">
-        <v>0.019242508810321413</v>
+        <v>0.019222587126321078</v>
       </c>
       <c r="I58">
-        <v>0.0017836493702624218</v>
+        <v>0.0013601473368735656</v>
       </c>
       <c r="J58">
-        <v>0.03775589018826164</v>
+        <v>0.03643059423991454</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -50896,39 +50896,39 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>corridor:58:nizi:kampala-uga</t>
+          <t>corridor:58:kilo:arua-uga</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>nizi</t>
+          <t>kilo</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>kampala-uga</t>
+          <t>arua-uga</t>
         </is>
       </c>
       <c r="D59">
         <v>30</v>
       </c>
       <c r="E59">
-        <v>0.0030397115334472313</v>
+        <v>0.0028404048325195996</v>
       </c>
       <c r="F59">
-        <v>0.007798503469288315</v>
+        <v>0.007786957767991598</v>
       </c>
       <c r="G59">
-        <v>0.007513934292532054</v>
+        <v>0.007030184083863106</v>
       </c>
       <c r="H59">
-        <v>0.01920949889117962</v>
+        <v>0.019202630017290306</v>
       </c>
       <c r="I59">
-        <v>0.0016678403853665758</v>
+        <v>0.0018407478578635922</v>
       </c>
       <c r="J59">
-        <v>0.03881661822899164</v>
+        <v>0.041169590401536636</v>
       </c>
       <c r="K59" t="inlineStr">
         <is>
@@ -50964,12 +50964,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>corridor:59:nizi:beni-cod</t>
+          <t>corridor:59:bambu:beni-cod</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>nizi</t>
+          <t>bambu</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -50981,22 +50981,22 @@
         <v>30</v>
       </c>
       <c r="E60">
-        <v>0.0028279586473544394</v>
+        <v>0.0030164649861187665</v>
       </c>
       <c r="F60">
-        <v>0.007773442977447614</v>
+        <v>0.007772299321732512</v>
       </c>
       <c r="G60">
-        <v>0.006991592151725234</v>
+        <v>0.0074649703248304</v>
       </c>
       <c r="H60">
-        <v>0.019148124794601235</v>
+        <v>0.01916669022271858</v>
       </c>
       <c r="I60">
-        <v>0.001626485696169075</v>
+        <v>0.0017745338814096486</v>
       </c>
       <c r="J60">
-        <v>0.04043085112899037</v>
+        <v>0.04144693368617039</v>
       </c>
       <c r="K60" t="inlineStr">
         <is>
@@ -51032,39 +51032,39 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>corridor:60:bambu:kasese-uga</t>
+          <t>corridor:60:miti-murhesa:kampala-uga</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>bambu</t>
+          <t>miti-murhesa</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>kasese-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D61">
         <v>30</v>
       </c>
       <c r="E61">
-        <v>0.0029787064606684455</v>
+        <v>0.002780055599183956</v>
       </c>
       <c r="F61">
-        <v>0.007727723579566553</v>
+        <v>0.0077543800748747505</v>
       </c>
       <c r="G61">
-        <v>0.007363466593160867</v>
+        <v>0.006881123372275866</v>
       </c>
       <c r="H61">
-        <v>0.01903614948937532</v>
+        <v>0.01912275597116167</v>
       </c>
       <c r="I61">
-        <v>0.002161627379220277</v>
+        <v>0.001731233807528232</v>
       </c>
       <c r="J61">
-        <v>0.040700080739514</v>
+        <v>0.03818702256228324</v>
       </c>
       <c r="K61" t="inlineStr">
         <is>
@@ -51100,39 +51100,39 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>corridor:61:butembo:nebbi-uga</t>
+          <t>corridor:61:goma-cod:beni-cod</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>butembo</t>
+          <t>goma-cod</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>beni-cod</t>
         </is>
       </c>
       <c r="D62">
         <v>30</v>
       </c>
       <c r="E62">
-        <v>0.002794253883045994</v>
+        <v>0.0026587921388565305</v>
       </c>
       <c r="F62">
-        <v>0.007726643785385345</v>
+        <v>0.007745510300115388</v>
       </c>
       <c r="G62">
-        <v>0.006908435854105138</v>
+        <v>0.006581566727665494</v>
       </c>
       <c r="H62">
-        <v>0.019033505698469483</v>
+        <v>0.0191010070867213</v>
       </c>
       <c r="I62">
-        <v>0.0017974249505340796</v>
+        <v>0.0015209453885095762</v>
       </c>
       <c r="J62">
-        <v>0.040761246701666295</v>
+        <v>0.040091153412378705</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -51168,39 +51168,39 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>corridor:62:kilo:arua-uga</t>
+          <t>corridor:62:nizi:kampala-uga</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>kilo</t>
+          <t>nizi</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>arua-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D63">
         <v>30</v>
       </c>
       <c r="E63">
-        <v>0.0027895356588024944</v>
+        <v>0.0027361329624540076</v>
       </c>
       <c r="F63">
-        <v>0.007708922084123715</v>
+        <v>0.0075987291180549255</v>
       </c>
       <c r="G63">
-        <v>0.0068967939985309645</v>
+        <v>0.006772627856763858</v>
       </c>
       <c r="H63">
-        <v>0.018990099864912985</v>
+        <v>0.018741077563372677</v>
       </c>
       <c r="I63">
-        <v>0.0013975388045409515</v>
+        <v>0.0013777102458249037</v>
       </c>
       <c r="J63">
-        <v>0.042391251021321644</v>
+        <v>0.043087769872402426</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -51236,39 +51236,39 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>corridor:63:kilo:bundibugyo-uga</t>
+          <t>corridor:63:nizi:kasese-uga</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>kilo</t>
+          <t>nizi</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>bundibugyo-uga</t>
+          <t>kasese-uga</t>
         </is>
       </c>
       <c r="D64">
         <v>30</v>
       </c>
       <c r="E64">
-        <v>0.0024745761411364142</v>
+        <v>0.0028258568215484003</v>
       </c>
       <c r="F64">
-        <v>0.007569959524086317</v>
+        <v>0.007552854340310916</v>
       </c>
       <c r="G64">
-        <v>0.00611952005219521</v>
+        <v>0.006994252131591605</v>
       </c>
       <c r="H64">
-        <v>0.01864970148957265</v>
+        <v>0.018628569089331942</v>
       </c>
       <c r="I64">
-        <v>0.001552318276025716</v>
+        <v>0.0018339497806420303</v>
       </c>
       <c r="J64">
-        <v>0.034976270348434146</v>
+        <v>0.0447125896493108</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -51304,12 +51304,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>corridor:64:miti-murhesa:bundibugyo-uga</t>
+          <t>corridor:64:butembo:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>miti-murhesa</t>
+          <t>butembo</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -51321,22 +51321,22 @@
         <v>30</v>
       </c>
       <c r="E65">
-        <v>0.0028359961308326576</v>
+        <v>0.002862546240653324</v>
       </c>
       <c r="F65">
-        <v>0.00756961435820569</v>
+        <v>0.0075168412354912895</v>
       </c>
       <c r="G65">
-        <v>0.007011421744851615</v>
+        <v>0.007084869280098771</v>
       </c>
       <c r="H65">
-        <v>0.018648855869933034</v>
+        <v>0.0185402409724002</v>
       </c>
       <c r="I65">
-        <v>0.0011273495847349967</v>
+        <v>0.0017601300993422223</v>
       </c>
       <c r="J65">
-        <v>0.037299073210084584</v>
+        <v>0.04281508413149316</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -51372,39 +51372,39 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>corridor:65:goma-cod:nebbi-uga</t>
+          <t>corridor:65:miti-murhesa:bundibugyo-uga</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>goma-cod</t>
+          <t>miti-murhesa</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>bundibugyo-uga</t>
         </is>
       </c>
       <c r="D66">
         <v>30</v>
       </c>
       <c r="E66">
-        <v>0.002833861264198795</v>
+        <v>0.002806475854065099</v>
       </c>
       <c r="F66">
-        <v>0.007547888001259828</v>
+        <v>0.007390944356303691</v>
       </c>
       <c r="G66">
-        <v>0.007006154836616929</v>
+        <v>0.006946382389732636</v>
       </c>
       <c r="H66">
-        <v>0.018595628743809794</v>
+        <v>0.018231416239954695</v>
       </c>
       <c r="I66">
-        <v>0.00218933896549888</v>
+        <v>0.00208300583836101</v>
       </c>
       <c r="J66">
-        <v>0.04012855964424418</v>
+        <v>0.03944316706094814</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -51440,39 +51440,39 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>corridor:66:nizi:nebbi-uga</t>
+          <t>corridor:66:kilo:kampala-uga</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>nizi</t>
+          <t>kilo</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>nebbi-uga</t>
+          <t>kampala-uga</t>
         </is>
       </c>
       <c r="D67">
         <v>30</v>
       </c>
       <c r="E67">
-        <v>0.0028713896563432317</v>
+        <v>0.0028636196069686815</v>
       </c>
       <c r="F67">
-        <v>0.007546538100174749</v>
+        <v>0.007245116575636645</v>
       </c>
       <c r="G67">
-        <v>0.007098739218278277</v>
+        <v>0.0070875198104265735</v>
       </c>
       <c r="H67">
-        <v>0.018592320839906473</v>
+        <v>0.017873638059777402</v>
       </c>
       <c r="I67">
-        <v>0.002009283025009237</v>
+        <v>0.001885099074969826</v>
       </c>
       <c r="J67">
-        <v>0.035894482626523734</v>
+        <v>0.04037313015728034</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -51983,10 +51983,10 @@
       </c>
       <c r="D9"/>
       <c r="E9">
-        <v>0.4036352802540115</v>
+        <v>0.4031809300428392</v>
       </c>
       <c r="F9">
-        <v>0.46215932894360784</v>
+        <v>0.4637985606142611</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -52037,10 +52037,10 @@
       </c>
       <c r="D10"/>
       <c r="E10">
-        <v>2.5636921180997643</v>
+        <v>2.658988714502407</v>
       </c>
       <c r="F10">
-        <v>12.502589644513742</v>
+        <v>12.09131304558839</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -52091,10 +52091,10 @@
       </c>
       <c r="D11"/>
       <c r="E11">
-        <v>455</v>
+        <v>468</v>
       </c>
       <c r="F11">
-        <v>725</v>
+        <v>712</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -52350,7 +52350,7 @@
         </is>
       </c>
       <c r="D16">
-        <v>0.003</v>
+        <v>0.008</v>
       </c>
       <c r="E16"/>
       <c r="F16"/>
@@ -52402,7 +52402,7 @@
         </is>
       </c>
       <c r="D17">
-        <v>0.018</v>
+        <v>0.019</v>
       </c>
       <c r="E17"/>
       <c r="F17"/>
@@ -52454,7 +52454,7 @@
         </is>
       </c>
       <c r="D18">
-        <v>0.979</v>
+        <v>0.973</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -52705,7 +52705,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>{"confirmation_backlog_50": [455, 725], "reporting_completeness_50": [0.4036352802540115, 0.46215932894360784]}</t>
+          <t>{"confirmation_backlog_50": [468, 712], "reporting_completeness_50": [0.4031809300428392, 0.4637985606142611]}</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -52734,12 +52734,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{"confirmed_endpoint": 112, "reporting_completeness_50": [0.4036352802540115, 0.46215932894360784]}</t>
+          <t>{"confirmed_endpoint": 112, "reporting_completeness_50": [0.4031809300428392, 0.4637985606142611]}</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>{"endpoint_confirmable_50": [242, 277]}</t>
+          <t>{"endpoint_confirmable_50": [241, 278]}</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">

</xml_diff>

<commit_message>
Fix Goma self-edge snapshot contract gate
</commit_message>
<xml_diff>
--- a/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
+++ b/deliverables/public-health-dataset/lovs-public-health-dataset.xlsx
@@ -1081,7 +1081,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>headline confirmed total 112; officially zone-attributed corridor source-load total 79 across 11 DRC MoH source zones; 33 confirmed cases remain unallocated headline context; current 66-corridor adjusted 50% range is 0.6-21.2% lower bounds and 1.8-48.2% upper bounds.</t>
+          <t>headline confirmed total 112; officially zone-attributed corridor source-load total 79 across 11 DRC MoH source zones; 33 confirmed cases remain unallocated headline context; current 76-corridor adjusted 50% range is 0.6-21.8% lower bounds and 1.8-49.4% upper bounds.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Ministere de la Sante Publique, Hygiene et Prevoyance sociale, Democratic Republic of the Congo. SitRep MVE N 007/MVB_17/2026 official PDF, cumulative Table IV, data as of 21 May 2026 / published 22 May 2026.; US CDC. Ebola Disease: Current Situation, 24 May 2026.; data/snapshot_contract.json generated from data/live-bdbv-2026-output.json by lovs/snapshot_contract.py.; lovs/lovs_next_zone.py source-load selection and corridor driver generation.; Evidence chain PUBLIC-CLAIM-AUDIT and public claim audit row BDBV-CLAIM-005.</t>
+          <t>Ministere de la Sante Publique, Hygiene et Prevoyance sociale, Democratic Republic of the Congo. SitRep MVE N 007/MVB_17/2026 official PDF, cumulative Table IV, data as of 21 May 2026 / published 22 May 2026.; US CDC. Ebola Disease: Current Situation, 25 May 2026.; data/snapshot_contract.json generated from data/live-bdbv-2026-output.json by lovs/snapshot_contract.py.; lovs/lovs_next_zone.py source-load selection and corridor driver generation.; Evidence chain PUBLIC-CLAIM-AUDIT and public claim audit row BDBV-CLAIM-005.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">

</xml_diff>